<commit_message>
fix(dev): hoja Meta propone presupuesto por ad set (igual que Google)
Cada ad set ahora tiene Spend actual, Accion, Spend propuesto, delta Spend
y delta % (mismo formato que la hoja Detalle Google).

Reglas Meta por CPR:
  CPR menor a 2 -> ESCALAR FUERTE x1.80
  CPR menor a 5 -> ESCALAR LEVE x1.30
  CPR 5-10 -> MANTENER x1.00
  CPR 10-20 -> RECORTAR x0.65
  CPR mayor a 20 -> RECORTAR FUERTE x0.40

Despues del factor se reescala al target Meta del seguro.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/suratech_propuesta_distribucion_mayo2026.xlsx
+++ b/outputs/suratech_propuesta_distribucion_mayo2026.xlsx
@@ -93,7 +93,8 @@
       <sz val="10"/>
     </font>
     <font>
-      <b val="1"/>
+      <name val="Calibri"/>
+      <color rgb="0053565A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -171,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -199,7 +200,9 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1652,17 +1655,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1675,7 +1681,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total: 21 ad sets · Fuente: export del Ads Manager</t>
+          <t>Total relevante: 19 ad sets en los 4 productos · Fuente: export del Ads Manager</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1708,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Spend (USD)</t>
+          <t>Spend actual</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1712,12 +1718,27 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
+          <t>Acción</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Spend propuesto</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Δ Spend</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Δ %</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
           <t>Estado</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Acción sugerida</t>
         </is>
       </c>
     </row>
@@ -1746,14 +1767,23 @@
           <t>actions:onsite_conversion.messaging_conversation_started_7d</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>ESCALAR FUERTE</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>670</v>
+      </c>
+      <c r="I5" s="18" t="n">
+        <v>211.02</v>
+      </c>
+      <c r="J5" s="25" t="n">
+        <v>0.459758595145758</v>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H5" s="17" t="inlineStr">
-        <is>
-          <t>ESCALAR FUERTE</t>
         </is>
       </c>
     </row>
@@ -1782,14 +1812,23 @@
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G6" s="11" t="inlineStr">
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>ESCALAR LEVE</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>830</v>
+      </c>
+      <c r="I6" s="18" t="n">
+        <v>42.69000000000005</v>
+      </c>
+      <c r="J6" s="25" t="n">
+        <v>0.05422260608908824</v>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H6" s="20" t="inlineStr">
-        <is>
-          <t>ESCALAR LEVE</t>
         </is>
       </c>
     </row>
@@ -1818,14 +1857,23 @@
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>ESCALAR LEVE</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>616</v>
+      </c>
+      <c r="I7" s="18" t="n">
+        <v>31.29999999999995</v>
+      </c>
+      <c r="J7" s="25" t="n">
+        <v>0.05353172567128434</v>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H7" s="20" t="inlineStr">
-        <is>
-          <t>ESCALAR LEVE</t>
         </is>
       </c>
     </row>
@@ -1854,14 +1902,23 @@
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G8" s="11" t="inlineStr">
+      <c r="G8" s="26" t="inlineStr">
+        <is>
+          <t>MANTENER</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>2144</v>
+      </c>
+      <c r="I8" s="18" t="n">
+        <v>-499.5100000000002</v>
+      </c>
+      <c r="J8" s="27" t="n">
+        <v>-0.188957106271586</v>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H8" s="25" t="inlineStr">
-        <is>
-          <t>MANTENER</t>
         </is>
       </c>
     </row>
@@ -1890,14 +1947,23 @@
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="G9" s="26" t="inlineStr">
+        <is>
+          <t>MANTENER</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>3275</v>
+      </c>
+      <c r="I9" s="18" t="n">
+        <v>-764.3699999999999</v>
+      </c>
+      <c r="J9" s="27" t="n">
+        <v>-0.189230003688694</v>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H9" s="25" t="inlineStr">
-        <is>
-          <t>MANTENER</t>
         </is>
       </c>
     </row>
@@ -1926,14 +1992,23 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.Lead_Autos_Di</t>
         </is>
       </c>
-      <c r="G10" s="11" t="inlineStr">
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>ESCALAR FUERTE</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="I10" s="18" t="n">
+        <v>10.48</v>
+      </c>
+      <c r="J10" s="25" t="n">
+        <v>0.8370607028753995</v>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
-        </is>
-      </c>
-      <c r="H10" s="17" t="inlineStr">
-        <is>
-          <t>ESCALAR FUERTE</t>
         </is>
       </c>
     </row>
@@ -1962,14 +2037,23 @@
           <t>actions:leadgen.other</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>ESCALAR LEVE</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>1146</v>
+      </c>
+      <c r="I11" s="18" t="n">
+        <v>264.4400000000001</v>
+      </c>
+      <c r="J11" s="25" t="n">
+        <v>0.2999682381233269</v>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H11" s="20" t="inlineStr">
-        <is>
-          <t>ESCALAR LEVE</t>
         </is>
       </c>
     </row>
@@ -1998,14 +2082,23 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G12" s="11" t="inlineStr">
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>ESCALAR LEVE</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>4679</v>
+      </c>
+      <c r="I12" s="18" t="n">
+        <v>1080.25</v>
+      </c>
+      <c r="J12" s="25" t="n">
+        <v>0.3001736714136853</v>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H12" s="20" t="inlineStr">
-        <is>
-          <t>ESCALAR LEVE</t>
         </is>
       </c>
     </row>
@@ -2034,14 +2127,23 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G13" s="11" t="inlineStr">
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>ESCALAR LEVE</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>5799</v>
+      </c>
+      <c r="I13" s="18" t="n">
+        <v>1338.6</v>
+      </c>
+      <c r="J13" s="25" t="n">
+        <v>0.3001076136669358</v>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H13" s="20" t="inlineStr">
-        <is>
-          <t>ESCALAR LEVE</t>
         </is>
       </c>
     </row>
@@ -2070,14 +2172,23 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G14" s="11" t="inlineStr">
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>ESCALAR LEVE</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="I14" s="18" t="n">
+        <v>238.29</v>
+      </c>
+      <c r="J14" s="25" t="n">
+        <v>0.2998452265606321</v>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H14" s="20" t="inlineStr">
-        <is>
-          <t>ESCALAR LEVE</t>
         </is>
       </c>
     </row>
@@ -2106,14 +2217,23 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="G15" s="26" t="inlineStr">
+        <is>
+          <t>MANTENER</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>878</v>
+      </c>
+      <c r="I15" s="18" t="n">
+        <v>0.5199999999999818</v>
+      </c>
+      <c r="J15" s="25" t="n">
+        <v>0.0005926060992842934</v>
+      </c>
+      <c r="K15" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H15" s="25" t="inlineStr">
-        <is>
-          <t>MANTENER</t>
         </is>
       </c>
     </row>
@@ -2142,14 +2262,23 @@
           <t>actions:leadgen.other</t>
         </is>
       </c>
-      <c r="G16" s="11" t="inlineStr">
+      <c r="G16" s="17" t="inlineStr">
+        <is>
+          <t>ESCALAR FUERTE</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>2596</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>1627.78</v>
+      </c>
+      <c r="J16" s="25" t="n">
+        <v>1.681208816178141</v>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H16" s="17" t="inlineStr">
-        <is>
-          <t>ESCALAR FUERTE</t>
         </is>
       </c>
     </row>
@@ -2178,14 +2307,23 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/MOTOS</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G17" s="22" t="inlineStr">
+        <is>
+          <t>RECORTAR</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>2561</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>-83.9699999999998</v>
+      </c>
+      <c r="J17" s="27" t="n">
+        <v>-0.03174705195143983</v>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H17" s="22" t="inlineStr">
-        <is>
-          <t>RECORTAR</t>
         </is>
       </c>
     </row>
@@ -2214,14 +2352,23 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/MOTOS</t>
         </is>
       </c>
-      <c r="G18" s="11" t="inlineStr">
+      <c r="G18" s="22" t="inlineStr">
+        <is>
+          <t>RECORTAR</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>3230</v>
+      </c>
+      <c r="I18" s="18" t="n">
+        <v>-105.4099999999999</v>
+      </c>
+      <c r="J18" s="27" t="n">
+        <v>-0.03160331113716151</v>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H18" s="22" t="inlineStr">
-        <is>
-          <t>RECORTAR</t>
         </is>
       </c>
     </row>
@@ -2250,14 +2397,23 @@
           <t>actions:onsite_conversion.messaging_conversation_started_7d</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>ESCALAR FUERTE</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>2068</v>
+      </c>
+      <c r="I19" s="18" t="n">
+        <v>1546.59</v>
+      </c>
+      <c r="J19" s="25" t="n">
+        <v>2.966168658061795</v>
+      </c>
+      <c r="K19" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H19" s="17" t="inlineStr">
-        <is>
-          <t>ESCALAR FUERTE</t>
         </is>
       </c>
     </row>
@@ -2286,14 +2442,23 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G20" s="11" t="inlineStr">
+      <c r="G20" s="23" t="inlineStr">
+        <is>
+          <t>RECORTAR FUERTE</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>1035</v>
+      </c>
+      <c r="I20" s="18" t="n">
+        <v>-139.25</v>
+      </c>
+      <c r="J20" s="27" t="n">
+        <v>-0.1185863317010858</v>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H20" s="23" t="inlineStr">
-        <is>
-          <t>RECORTAR FUERTE</t>
         </is>
       </c>
     </row>
@@ -2322,14 +2487,23 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="G21" s="23" t="inlineStr">
+        <is>
+          <t>RECORTAR FUERTE</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>1027</v>
+      </c>
+      <c r="I21" s="18" t="n">
+        <v>-137.9000000000001</v>
+      </c>
+      <c r="J21" s="27" t="n">
+        <v>-0.1183792600223196</v>
+      </c>
+      <c r="K21" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H21" s="23" t="inlineStr">
-        <is>
-          <t>RECORTAR FUERTE</t>
         </is>
       </c>
     </row>
@@ -2358,14 +2532,23 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G22" s="11" t="inlineStr">
+      <c r="G22" s="23" t="inlineStr">
+        <is>
+          <t>RECORTAR FUERTE</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>211</v>
+      </c>
+      <c r="I22" s="18" t="n">
+        <v>-28.21000000000001</v>
+      </c>
+      <c r="J22" s="27" t="n">
+        <v>-0.1179298524309185</v>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H22" s="23" t="inlineStr">
-        <is>
-          <t>RECORTAR FUERTE</t>
         </is>
       </c>
     </row>
@@ -2394,21 +2577,30 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="G23" s="23" t="inlineStr">
+        <is>
+          <t>RECORTAR FUERTE</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>214</v>
+      </c>
+      <c r="I23" s="18" t="n">
+        <v>-29.03</v>
+      </c>
+      <c r="J23" s="27" t="n">
+        <v>-0.1194502736287701</v>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="H23" s="23" t="inlineStr">
-        <is>
-          <t>RECORTAR FUERTE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>Agregado Meta por seguro</t>
+          <t>Total Meta por seguro</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2647,7 @@
           <t>Auto</t>
         </is>
       </c>
-      <c r="B28" s="26" t="n">
+      <c r="B28" s="28" t="n">
         <v>6</v>
       </c>
       <c r="C28" s="5" t="n">
@@ -2480,7 +2672,7 @@
           <t>Moto</t>
         </is>
       </c>
-      <c r="B29" s="26" t="n">
+      <c r="B29" s="28" t="n">
         <v>3</v>
       </c>
       <c r="C29" s="5" t="n">
@@ -2505,7 +2697,7 @@
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="B30" s="26" t="n">
+      <c r="B30" s="28" t="n">
         <v>5</v>
       </c>
       <c r="C30" s="5" t="n">
@@ -2530,7 +2722,7 @@
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B31" s="26" t="n">
+      <c r="B31" s="28" t="n">
         <v>5</v>
       </c>
       <c r="C31" s="5" t="n">
@@ -2543,16 +2735,16 @@
         <v>3.824713958810069</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>4554</v>
+        <v>4555</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>1211.2</v>
+        <v>1212.2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2579,208 +2771,208 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="27" t="inlineStr">
+      <c r="A3" s="29" t="inlineStr">
         <is>
           <t>Datos base</t>
         </is>
       </c>
-      <c r="B3" s="28" t="inlineStr">
+      <c r="B3" s="30" t="inlineStr">
         <is>
           <t>Performance real del 1-27 abril 2026 cruzado con Sheet Leads CRM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Constraint 1</t>
         </is>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Tope por seguro provisto por el cliente (Auto $52.421, Moto $32.642, Arriendo $31.080, Viajes $16.900)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Constraint 2</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>70-75% del presupuesto en Google (mejor calidad de leads SF según cliente)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Constraint 3</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>Bing se mantiene en presupuesto del Flow</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="inlineStr"/>
-      <c r="B7" s="28" t="inlineStr"/>
+      <c r="A7" s="31" t="inlineStr"/>
+      <c r="B7" s="30" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>Reglas de clasificación de campañas Google</t>
         </is>
       </c>
-      <c r="B8" s="28" t="inlineStr"/>
+      <c r="B8" s="30" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE (×1.80)</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>CPA ≤ $7 y % Lost Budget ≥ 50% — palanca #1</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>ESCALAR (×1.40)</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="30" t="inlineStr">
         <is>
           <t>CPA ≤ $10 y % Lost Budget ≥ 30%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>ESCALAR LEVE (×1.20)</t>
         </is>
       </c>
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B11" s="30" t="inlineStr">
         <is>
           <t>CPA ≤ $10 y % Lost Budget ≥ 10%</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>ESCALAR MODERADO (×1.20)</t>
         </is>
       </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="30" t="inlineStr">
         <is>
           <t>CPA ≤ $15 y % Lost Budget ≥ 50%</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>RECORTAR (×0.65)</t>
         </is>
       </c>
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="30" t="inlineStr">
         <is>
           <t>CPA entre $15 y $25</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE (×0.40)</t>
         </is>
       </c>
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>CPA &gt; $25</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>MANTENER (×1.00)</t>
         </is>
       </c>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>Resto</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr"/>
-      <c r="B16" s="28" t="inlineStr"/>
+      <c r="A16" s="31" t="inlineStr"/>
+      <c r="B16" s="30" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="27" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>Ajuste fino</t>
         </is>
       </c>
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>Después del factor inicial, los presupuestos de Google se reescalan proporcionalmente para alcanzar exactamente el 72% del total por seguro.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="inlineStr"/>
-      <c r="B18" s="28" t="inlineStr"/>
+      <c r="A18" s="31" t="inlineStr"/>
+      <c r="B18" s="30" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>Limitaciones honestas</t>
         </is>
       </c>
-      <c r="B19" s="28" t="inlineStr"/>
+      <c r="B19" s="30" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
+      <c r="A20" s="29" t="inlineStr">
         <is>
           <t>Meta</t>
         </is>
       </c>
-      <c r="B20" s="28" t="inlineStr">
+      <c r="B20" s="30" t="inlineStr">
         <is>
           <t>Detalle por ad set requiere CSV exportado del Ads Manager (Reports → Export Reports). Esta propuesta optimiza Meta a nivel seguro.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="inlineStr">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>Bing</t>
         </is>
       </c>
-      <c r="B21" s="28" t="inlineStr">
+      <c r="B21" s="30" t="inlineStr">
         <is>
           <t>No se modificó (sin acceso desde el extractor).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
+      <c r="A22" s="29" t="inlineStr">
         <is>
           <t>Estacionalidad</t>
         </is>
       </c>
-      <c r="B22" s="28" t="inlineStr">
+      <c r="B22" s="30" t="inlineStr">
         <is>
           <t>Asume ritmo similar a abril. Si hay cambios estacionales, ajustar.</t>
         </is>

</xml_diff>

<commit_message>
fix(dev): justificacion ahora se genera correctamente (campos opcionales con .get())
</commit_message>
<xml_diff>
--- a/outputs/suratech_propuesta_distribucion_mayo2026.xlsx
+++ b/outputs/suratech_propuesta_distribucion_mayo2026.xlsx
@@ -172,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -189,21 +189,64 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -987,20 +1030,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1066,584 +1110,659 @@
           <t>Δ %</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Justificación</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>SURA_AUTOS_PMAX</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
+      <c r="C4" s="16" t="n">
         <v>3.9</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="17" t="n">
         <v>0.74</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="18" t="n">
         <v>517</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="18" t="n">
         <v>10672</v>
       </c>
-      <c r="G4" s="16" t="n">
+      <c r="G4" s="19" t="n">
         <v>2739.4</v>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="H4" s="20" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE</t>
         </is>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="18" t="n">
         <v>19331</v>
       </c>
-      <c r="J4" s="18" t="n">
+      <c r="J4" s="21" t="n">
         <v>8659</v>
       </c>
-      <c r="K4" s="19" t="n">
-        <v>81.13755622188906</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="K4" s="22" t="n">
+        <v>0.8113755622188905</v>
+      </c>
+      <c r="L4" s="23" t="inlineStr">
+        <is>
+          <t>CPA $3.90 excelente y pierde 74% de impresiones por presupuesto. Subir budget convierte impresiones perdidas en conversiones al mismo CPA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>SURA_AUTOS_SEARCH_SEGMENT</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C5" s="16" t="n">
         <v>6.72</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="18" t="n">
         <v>326</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="18" t="n">
         <v>9198</v>
       </c>
-      <c r="G5" s="16" t="n">
+      <c r="G5" s="19" t="n">
         <v>1369.1</v>
       </c>
-      <c r="H5" s="20" t="inlineStr">
+      <c r="H5" s="24" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="18" t="n">
         <v>11107</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="J5" s="21" t="n">
         <v>1909</v>
       </c>
-      <c r="K5" s="19" t="n">
-        <v>20.75451185040226</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="K5" s="22" t="n">
+        <v>0.2075451185040226</v>
+      </c>
+      <c r="L5" s="23" t="inlineStr">
+        <is>
+          <t>CPA $6.72, 1,369 conversiones ya validan el formato, 15% lost budget = headroom. Subir budget para capitalizar la eficiencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>SURA_AUTOS_SEARCH_RETENTION</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="16" t="n">
         <v>10.59</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="17" t="n">
         <v>0.23</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="18" t="n">
         <v>147</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="18" t="n">
         <v>4194</v>
       </c>
-      <c r="G6" s="16" t="n">
+      <c r="G6" s="19" t="n">
         <v>396.1</v>
       </c>
-      <c r="H6" s="21" t="inlineStr">
+      <c r="H6" s="25" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="I6" s="18" t="n">
         <v>4220</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="21" t="n">
         <v>26</v>
       </c>
-      <c r="K6" s="19" t="n">
-        <v>0.619933237958989</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="K6" s="22" t="n">
+        <v>0.00619933237958989</v>
+      </c>
+      <c r="L6" s="23" t="inlineStr">
+        <is>
+          <t>CPA $10.59. Monitorear y mantener estable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>SURA_AUTOS_SEARCH_CONQUEST</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="16" t="n">
         <v>6.41</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="17" t="n">
         <v>0.42</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="18" t="n">
         <v>52</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="18" t="n">
         <v>2189</v>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="G7" s="19" t="n">
         <v>341.7</v>
       </c>
-      <c r="H7" s="20" t="inlineStr">
+      <c r="H7" s="24" t="inlineStr">
         <is>
           <t>ESCALAR</t>
         </is>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="I7" s="18" t="n">
         <v>3084</v>
       </c>
-      <c r="J7" s="18" t="n">
+      <c r="J7" s="21" t="n">
         <v>895</v>
       </c>
-      <c r="K7" s="19" t="n">
-        <v>40.886249428963</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="K7" s="22" t="n">
+        <v>0.40886249428963</v>
+      </c>
+      <c r="L7" s="23" t="inlineStr">
+        <is>
+          <t>CPA $6.41, 341 conversiones ya validan el formato, 42% lost budget = headroom. Subir budget para capitalizar la eficiencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Moto</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>SURA_MOTOS_SEARCH_RETENTION</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="16" t="n">
         <v>6.46</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="17" t="n">
         <v>0.04</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="18" t="n">
         <v>183</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="18" t="n">
         <v>1994</v>
       </c>
-      <c r="G9" s="16" t="n">
+      <c r="G9" s="19" t="n">
         <v>308.8</v>
       </c>
-      <c r="H9" s="21" t="inlineStr">
+      <c r="H9" s="25" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="I9" s="18" t="n">
         <v>2926</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J9" s="21" t="n">
         <v>932</v>
       </c>
-      <c r="K9" s="19" t="n">
-        <v>46.74022066198596</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="K9" s="22" t="n">
+        <v>0.4674022066198596</v>
+      </c>
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>CPA $6.46 aceptable y la campaña ya consume su budget (lost 4%). Sin headroom para escalar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Moto</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>SURA_MOTOS_PMAX</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="16" t="n">
         <v>12.19</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="17" t="n">
         <v>0.58</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="18" t="n">
         <v>397</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="18" t="n">
         <v>7832</v>
       </c>
-      <c r="G10" s="16" t="n">
+      <c r="G10" s="19" t="n">
         <v>642.7</v>
       </c>
-      <c r="H10" s="20" t="inlineStr">
+      <c r="H10" s="24" t="inlineStr">
         <is>
           <t>ESCALAR MODERADO</t>
         </is>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="I10" s="18" t="n">
         <v>13789</v>
       </c>
-      <c r="J10" s="18" t="n">
+      <c r="J10" s="21" t="n">
         <v>5957</v>
       </c>
-      <c r="K10" s="19" t="n">
-        <v>76.05975485188968</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="K10" s="22" t="n">
+        <v>0.7605975485188968</v>
+      </c>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>CPA $12.19, 642 conversiones ya validan el formato, 58% lost budget = headroom. Subir budget para capitalizar la eficiencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Moto</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>SURA_MOTOS_SEARCH_SEGMENT</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="16" t="n">
         <v>15.66</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="17" t="n">
         <v>0.66</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="18" t="n">
         <v>357</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="18" t="n">
         <v>4596</v>
       </c>
-      <c r="G11" s="16" t="n">
+      <c r="G11" s="19" t="n">
         <v>293.5</v>
       </c>
-      <c r="H11" s="22" t="inlineStr">
+      <c r="H11" s="26" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="I11" s="18" t="n">
         <v>4383</v>
       </c>
-      <c r="J11" s="18" t="n">
+      <c r="J11" s="21" t="n">
         <v>-213</v>
       </c>
-      <c r="K11" s="19" t="n">
-        <v>-4.634464751958225</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="K11" s="22" t="n">
+        <v>-0.04634464751958225</v>
+      </c>
+      <c r="L11" s="23" t="inlineStr">
+        <is>
+          <t>CPA $15.66 alto + tiene anuncios rechazados. Recortar mientras se corrigen los assets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Moto</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>SURA_MOTOS_SEARCH_CONQUEST</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="17" t="n">
         <v>0.73</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="18" t="n">
         <v>75</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="18" t="n">
         <v>1366</v>
       </c>
-      <c r="G12" s="16" t="n">
+      <c r="G12" s="19" t="n">
         <v>97.59999999999999</v>
       </c>
-      <c r="H12" s="20" t="inlineStr">
+      <c r="H12" s="24" t="inlineStr">
         <is>
           <t>ESCALAR MODERADO</t>
         </is>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="I12" s="18" t="n">
         <v>2405</v>
       </c>
-      <c r="J12" s="18" t="n">
+      <c r="J12" s="21" t="n">
         <v>1039</v>
       </c>
-      <c r="K12" s="19" t="n">
-        <v>76.0614934114202</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="K12" s="22" t="n">
+        <v>0.760614934114202</v>
+      </c>
+      <c r="L12" s="23" t="inlineStr">
+        <is>
+          <t>CPA $14.00, 73% lost budget = headroom. Subir budget para capitalizar la eficiencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>sura-cdd-co-google-search-retention-arriendo</t>
         </is>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="16" t="n">
         <v>7.32</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="17" t="n">
         <v>0.06</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="18" t="n">
         <v>984</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="18" t="n">
         <v>12383</v>
       </c>
-      <c r="G14" s="16" t="n">
+      <c r="G14" s="19" t="n">
         <v>1690.7</v>
       </c>
-      <c r="H14" s="21" t="inlineStr">
+      <c r="H14" s="25" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="I14" s="18" t="n">
         <v>13603</v>
       </c>
-      <c r="J14" s="18" t="n">
+      <c r="J14" s="21" t="n">
         <v>1220</v>
       </c>
-      <c r="K14" s="19" t="n">
-        <v>9.852216748768473</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="K14" s="22" t="n">
+        <v>0.09852216748768473</v>
+      </c>
+      <c r="L14" s="23" t="inlineStr">
+        <is>
+          <t>CPA $7.32 aceptable y la campaña ya consume su budget (lost 6%). Sin headroom para escalar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>SURA_ARRIENDO_SEARCH_SEGMENT</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="16" t="n">
         <v>25.27</v>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="17" t="n">
         <v>0.14</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="18" t="n">
         <v>900</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="18" t="n">
         <v>8208</v>
       </c>
-      <c r="G15" s="16" t="n">
+      <c r="G15" s="19" t="n">
         <v>324.8</v>
       </c>
-      <c r="H15" s="23" t="inlineStr">
+      <c r="H15" s="27" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE</t>
         </is>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="I15" s="18" t="n">
         <v>3606</v>
       </c>
-      <c r="J15" s="18" t="n">
+      <c r="J15" s="21" t="n">
         <v>-4602</v>
       </c>
-      <c r="K15" s="19" t="n">
-        <v>-56.0672514619883</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="K15" s="22" t="n">
+        <v>-0.560672514619883</v>
+      </c>
+      <c r="L15" s="23" t="inlineStr">
+        <is>
+          <t>CPA $25.27 insostenible. $8,208 invertidos generaron solo 324 conversiones. Bajar budget y revisar keywords/creatividades antes de seguir gastando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>SURA_ARRIENDO_PMAX</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
+      <c r="C16" s="16" t="n">
         <v>23.55</v>
       </c>
-      <c r="D16" s="15" t="n">
+      <c r="D16" s="17" t="n">
         <v>0.73</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="18" t="n">
         <v>376</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" s="18" t="n">
         <v>7238</v>
       </c>
-      <c r="G16" s="16" t="n">
+      <c r="G16" s="19" t="n">
         <v>307.3</v>
       </c>
-      <c r="H16" s="22" t="inlineStr">
+      <c r="H16" s="26" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="I16" s="18" t="n">
         <v>5169</v>
       </c>
-      <c r="J16" s="18" t="n">
+      <c r="J16" s="21" t="n">
         <v>-2069</v>
       </c>
-      <c r="K16" s="19" t="n">
-        <v>-28.58524454269135</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="K16" s="22" t="n">
+        <v>-0.2858524454269135</v>
+      </c>
+      <c r="L16" s="23" t="inlineStr">
+        <is>
+          <t>CPA $23.55 fuera de rango. Recortar y mover budget a campañas más eficientes del seguro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="50" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>SURA_VIAJES_SEARCH_RETENTION</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
+      <c r="C18" s="16" t="n">
         <v>22.67</v>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="D18" s="17" t="n">
         <v>0.2</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E18" s="18" t="n">
         <v>251</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="18" t="n">
         <v>2971</v>
       </c>
-      <c r="G18" s="16" t="n">
+      <c r="G18" s="19" t="n">
         <v>131</v>
       </c>
-      <c r="H18" s="22" t="inlineStr">
+      <c r="H18" s="26" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="I18" s="18" t="n">
         <v>6003</v>
       </c>
-      <c r="J18" s="18" t="n">
+      <c r="J18" s="21" t="n">
         <v>3032</v>
       </c>
-      <c r="K18" s="19" t="n">
-        <v>102.0531807472232</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="K18" s="22" t="n">
+        <v>1.020531807472232</v>
+      </c>
+      <c r="L18" s="23" t="inlineStr">
+        <is>
+          <t>CPA $22.67 fuera de rango. Recortar y mover budget a campañas más eficientes del seguro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="50" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>SURA_VIAJES_PMAX</t>
         </is>
       </c>
-      <c r="C19" s="14" t="n">
+      <c r="C19" s="16" t="n">
         <v>20.66</v>
       </c>
-      <c r="D19" s="15" t="n">
+      <c r="D19" s="17" t="n">
         <v>0.77</v>
       </c>
-      <c r="E19" s="5" t="n">
+      <c r="E19" s="18" t="n">
         <v>155</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="18" t="n">
         <v>1959</v>
       </c>
-      <c r="G19" s="16" t="n">
+      <c r="G19" s="19" t="n">
         <v>94.8</v>
       </c>
-      <c r="H19" s="22" t="inlineStr">
+      <c r="H19" s="26" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="I19" s="18" t="n">
         <v>3958</v>
       </c>
-      <c r="J19" s="18" t="n">
+      <c r="J19" s="21" t="n">
         <v>1999</v>
       </c>
-      <c r="K19" s="19" t="n">
-        <v>102.0418580908627</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="K19" s="22" t="n">
+        <v>1.020418580908627</v>
+      </c>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>CPA $20.66 fuera de rango. Recortar y mover budget a campañas más eficientes del seguro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>SURA_VIAJES_SEARCH_SEGMENT</t>
         </is>
       </c>
-      <c r="C20" s="14" t="n">
+      <c r="C20" s="16" t="n">
         <v>54.52</v>
       </c>
-      <c r="D20" s="15" t="n">
+      <c r="D20" s="17" t="n">
         <v>0.58</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="18" t="n">
         <v>106</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="18" t="n">
         <v>1775</v>
       </c>
-      <c r="G20" s="16" t="n">
+      <c r="G20" s="19" t="n">
         <v>32.5</v>
       </c>
-      <c r="H20" s="23" t="inlineStr">
+      <c r="H20" s="27" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE</t>
         </is>
       </c>
-      <c r="I20" s="5" t="n">
+      <c r="I20" s="18" t="n">
         <v>2207</v>
       </c>
-      <c r="J20" s="18" t="n">
+      <c r="J20" s="21" t="n">
         <v>432</v>
       </c>
-      <c r="K20" s="19" t="n">
-        <v>24.33802816901408</v>
+      <c r="K20" s="22" t="n">
+        <v>0.2433802816901408</v>
+      </c>
+      <c r="L20" s="23" t="inlineStr">
+        <is>
+          <t>CPA $54.52 insostenible. $1,775 invertidos generaron solo 32 conversiones. Bajar budget y revisar keywords/creatividades antes de seguir gastando.</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1655,7 +1774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1669,6 +1788,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1741,859 +1861,959 @@
           <t>Estado</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Justificación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Mensajes_WHATSAPP_ARRIENDO_2026</t>
         </is>
       </c>
-      <c r="C5" s="24" t="n">
+      <c r="C5" s="28" t="n">
         <v>650</v>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="16" t="n">
         <v>0.70612308</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="18" t="n">
         <v>458.98</v>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>actions:onsite_conversion.messaging_conversation_started_7d</t>
         </is>
       </c>
-      <c r="G5" s="17" t="inlineStr">
+      <c r="G5" s="20" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="18" t="n">
         <v>670</v>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="I5" s="21" t="n">
         <v>211.02</v>
       </c>
-      <c r="J5" s="25" t="n">
+      <c r="J5" s="29" t="n">
         <v>0.459758595145758</v>
       </c>
-      <c r="K5" s="11" t="inlineStr">
+      <c r="K5" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="L5" s="23" t="inlineStr">
+        <is>
+          <t>CPR $0.71 excepcional (650 conversaciones WhatsApp). Es un outlier eficiente del MCC - vale la pena duplicar inversión y dejar que escale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_ARRIENDO_LISTA_RECOMPRA</t>
         </is>
       </c>
-      <c r="C6" s="24" t="n">
+      <c r="C6" s="28" t="n">
         <v>180</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="16" t="n">
         <v>4.37394444</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="18" t="n">
         <v>787.3099999999999</v>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="G6" s="24" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="18" t="n">
         <v>830</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="I6" s="21" t="n">
         <v>42.69000000000005</v>
       </c>
-      <c r="J6" s="25" t="n">
+      <c r="J6" s="29" t="n">
         <v>0.05422260608908824</v>
       </c>
-      <c r="K6" s="11" t="inlineStr">
+      <c r="K6" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="L6" s="23" t="inlineStr">
+        <is>
+          <t>CPR $4.37 bueno con 180 conversiones web validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_ARRIENDO_USUARIOS_SIN_INQUILINO_V2</t>
         </is>
       </c>
-      <c r="C7" s="24" t="n">
+      <c r="C7" s="28" t="n">
         <v>124</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="16" t="n">
         <v>4.71532258</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="18" t="n">
         <v>584.7</v>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G7" s="20" t="inlineStr">
+      <c r="G7" s="24" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="18" t="n">
         <v>616</v>
       </c>
-      <c r="I7" s="18" t="n">
+      <c r="I7" s="21" t="n">
         <v>31.29999999999995</v>
       </c>
-      <c r="J7" s="25" t="n">
+      <c r="J7" s="29" t="n">
         <v>0.05353172567128434</v>
       </c>
-      <c r="K7" s="11" t="inlineStr">
+      <c r="K7" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="L7" s="23" t="inlineStr">
+        <is>
+          <t>CPR $4.72 bueno con 124 conversiones web validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_ARRIENDO_RMKT_2025</t>
         </is>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="28" t="n">
         <v>522</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="16" t="n">
         <v>5.0641954</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="18" t="n">
         <v>2643.51</v>
       </c>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G8" s="26" t="inlineStr">
+      <c r="G8" s="30" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="18" t="n">
         <v>2144</v>
       </c>
-      <c r="I8" s="18" t="n">
+      <c r="I8" s="21" t="n">
         <v>-499.5100000000002</v>
       </c>
-      <c r="J8" s="27" t="n">
+      <c r="J8" s="31" t="n">
         <v>-0.188957106271586</v>
       </c>
-      <c r="K8" s="11" t="inlineStr">
+      <c r="K8" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>CPR $5.06 aceptable. 522 conversiones web. Mantener para no romper aprendizaje del algoritmo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_ARRIENDO_INTERESES_2025</t>
         </is>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="28" t="n">
         <v>741</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="16" t="n">
         <v>5.45124157</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="18" t="n">
         <v>4039.37</v>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G9" s="26" t="inlineStr">
+      <c r="G9" s="30" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="18" t="n">
         <v>3275</v>
       </c>
-      <c r="I9" s="18" t="n">
+      <c r="I9" s="21" t="n">
         <v>-764.3699999999999</v>
       </c>
-      <c r="J9" s="27" t="n">
+      <c r="J9" s="31" t="n">
         <v>-0.189230003688694</v>
       </c>
-      <c r="K9" s="11" t="inlineStr">
+      <c r="K9" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>CPR $5.45 aceptable. 741 conversiones web. Mantener para no romper aprendizaje del algoritmo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_AUTO_PLAN_GLOBAL_INTERESES_2025</t>
         </is>
       </c>
-      <c r="C10" s="24" t="n">
+      <c r="C10" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="16" t="n">
         <v>1.78857143</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="18" t="n">
         <v>12.52</v>
       </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="F10" s="15" t="inlineStr">
         <is>
           <t>conversions:offsite_conversion.fb_pixel_custom.Lead_Autos_Di</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
+      <c r="G10" s="20" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE</t>
         </is>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="18" t="n">
         <v>23</v>
       </c>
-      <c r="I10" s="18" t="n">
+      <c r="I10" s="21" t="n">
         <v>10.48</v>
       </c>
-      <c r="J10" s="25" t="n">
+      <c r="J10" s="29" t="n">
         <v>0.8370607028753995</v>
       </c>
-      <c r="K10" s="11" t="inlineStr">
+      <c r="K10" s="15" t="inlineStr">
         <is>
           <t>inactive</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>CPR $1.79 excepcional (7 conversiones web). Es un outlier eficiente del MCC - vale la pena duplicar inversión y dejar que escale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Clientes potenciales - Auto</t>
         </is>
       </c>
-      <c r="C11" s="24" t="n">
+      <c r="C11" s="28" t="n">
         <v>289</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="16" t="n">
         <v>3.05038062</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="18" t="n">
         <v>881.5599999999999</v>
       </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>actions:leadgen.other</t>
         </is>
       </c>
-      <c r="G11" s="20" t="inlineStr">
+      <c r="G11" s="24" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="18" t="n">
         <v>1146</v>
       </c>
-      <c r="I11" s="18" t="n">
+      <c r="I11" s="21" t="n">
         <v>264.4400000000001</v>
       </c>
-      <c r="J11" s="25" t="n">
+      <c r="J11" s="29" t="n">
         <v>0.2999682381233269</v>
       </c>
-      <c r="K11" s="11" t="inlineStr">
+      <c r="K11" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="L11" s="23" t="inlineStr">
+        <is>
+          <t>CPR $3.05 bueno con 289 leads (form) validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_AUTO_INTERESES_2025</t>
         </is>
       </c>
-      <c r="C12" s="24" t="n">
+      <c r="C12" s="28" t="n">
         <v>907</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="16" t="n">
         <v>3.96775083</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="18" t="n">
         <v>3598.75</v>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F12" s="15" t="inlineStr">
         <is>
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G12" s="20" t="inlineStr">
+      <c r="G12" s="24" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="18" t="n">
         <v>4679</v>
       </c>
-      <c r="I12" s="18" t="n">
+      <c r="I12" s="21" t="n">
         <v>1080.25</v>
       </c>
-      <c r="J12" s="25" t="n">
+      <c r="J12" s="29" t="n">
         <v>0.3001736714136853</v>
       </c>
-      <c r="K12" s="11" t="inlineStr">
+      <c r="K12" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="L12" s="23" t="inlineStr">
+        <is>
+          <t>CPR $3.97 bueno con 907 conversiones web validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_AUTO_RMKT_2025</t>
         </is>
       </c>
-      <c r="C13" s="24" t="n">
+      <c r="C13" s="28" t="n">
         <v>1083</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="16" t="n">
         <v>4.11855956</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="18" t="n">
         <v>4460.4</v>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F13" s="15" t="inlineStr">
         <is>
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G13" s="20" t="inlineStr">
+      <c r="G13" s="24" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="H13" s="18" t="n">
         <v>5799</v>
       </c>
-      <c r="I13" s="18" t="n">
+      <c r="I13" s="21" t="n">
         <v>1338.6</v>
       </c>
-      <c r="J13" s="25" t="n">
+      <c r="J13" s="29" t="n">
         <v>0.3001076136669358</v>
       </c>
-      <c r="K13" s="11" t="inlineStr">
+      <c r="K13" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="L13" s="23" t="inlineStr">
+        <is>
+          <t>CPR $4.12 bueno con 1,083 conversiones web validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_AUTO_INTERESES_PROMOCIONES</t>
         </is>
       </c>
-      <c r="C14" s="24" t="n">
+      <c r="C14" s="28" t="n">
         <v>176</v>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="16" t="n">
         <v>4.51539773</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="18" t="n">
         <v>794.71</v>
       </c>
-      <c r="F14" s="11" t="inlineStr">
+      <c r="F14" s="15" t="inlineStr">
         <is>
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G14" s="20" t="inlineStr">
+      <c r="G14" s="24" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="18" t="n">
         <v>1033</v>
       </c>
-      <c r="I14" s="18" t="n">
+      <c r="I14" s="21" t="n">
         <v>238.29</v>
       </c>
-      <c r="J14" s="25" t="n">
+      <c r="J14" s="29" t="n">
         <v>0.2998452265606321</v>
       </c>
-      <c r="K14" s="11" t="inlineStr">
+      <c r="K14" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="L14" s="23" t="inlineStr">
+        <is>
+          <t>CPR $4.52 bueno con 176 conversiones web validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_AUTO_RMKT_PROMOCIONES</t>
         </is>
       </c>
-      <c r="C15" s="24" t="n">
+      <c r="C15" s="28" t="n">
         <v>157</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="16" t="n">
         <v>5.58904459</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="18" t="n">
         <v>877.48</v>
       </c>
-      <c r="F15" s="11" t="inlineStr">
+      <c r="F15" s="15" t="inlineStr">
         <is>
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G15" s="26" t="inlineStr">
+      <c r="G15" s="30" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H15" s="18" t="n">
         <v>878</v>
       </c>
-      <c r="I15" s="18" t="n">
+      <c r="I15" s="21" t="n">
         <v>0.5199999999999818</v>
       </c>
-      <c r="J15" s="25" t="n">
+      <c r="J15" s="29" t="n">
         <v>0.0005926060992842934</v>
       </c>
-      <c r="K15" s="11" t="inlineStr">
+      <c r="K15" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="L15" s="23" t="inlineStr">
+        <is>
+          <t>CPR $5.59 aceptable. 157 conversiones web. Mantener para no romper aprendizaje del algoritmo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Moto</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>Clientes potenciales - Moto</t>
         </is>
       </c>
-      <c r="C16" s="24" t="n">
+      <c r="C16" s="28" t="n">
         <v>669</v>
       </c>
-      <c r="D16" s="14" t="n">
+      <c r="D16" s="16" t="n">
         <v>1.44726457</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="18" t="n">
         <v>968.22</v>
       </c>
-      <c r="F16" s="11" t="inlineStr">
+      <c r="F16" s="15" t="inlineStr">
         <is>
           <t>actions:leadgen.other</t>
         </is>
       </c>
-      <c r="G16" s="17" t="inlineStr">
+      <c r="G16" s="20" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE</t>
         </is>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="H16" s="18" t="n">
         <v>2596</v>
       </c>
-      <c r="I16" s="18" t="n">
+      <c r="I16" s="21" t="n">
         <v>1627.78</v>
       </c>
-      <c r="J16" s="25" t="n">
+      <c r="J16" s="29" t="n">
         <v>1.681208816178141</v>
       </c>
-      <c r="K16" s="11" t="inlineStr">
+      <c r="K16" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="L16" s="23" t="inlineStr">
+        <is>
+          <t>CPR $1.45 excepcional (669 leads (form)). Es un outlier eficiente del MCC - vale la pena duplicar inversión y dejar que escale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Moto</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_MOTO_INTERESES_2025</t>
         </is>
       </c>
-      <c r="C17" s="24" t="n">
+      <c r="C17" s="28" t="n">
         <v>256</v>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="D17" s="16" t="n">
         <v>10.33191406</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="18" t="n">
         <v>2644.97</v>
       </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="F17" s="15" t="inlineStr">
         <is>
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/MOTOS</t>
         </is>
       </c>
-      <c r="G17" s="22" t="inlineStr">
+      <c r="G17" s="26" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="H17" s="18" t="n">
         <v>2561</v>
       </c>
-      <c r="I17" s="18" t="n">
+      <c r="I17" s="21" t="n">
         <v>-83.9699999999998</v>
       </c>
-      <c r="J17" s="27" t="n">
+      <c r="J17" s="31" t="n">
         <v>-0.03174705195143983</v>
       </c>
-      <c r="K17" s="11" t="inlineStr">
+      <c r="K17" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="L17" s="23" t="inlineStr">
+        <is>
+          <t>CPR $10.33 arriba del rango eficiente del producto. Bajar budget y mover el spend a los ad sets que mejor convierten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="50" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Moto</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_MOTO_RMKT_2025</t>
         </is>
       </c>
-      <c r="C18" s="24" t="n">
+      <c r="C18" s="28" t="n">
         <v>312</v>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="D18" s="16" t="n">
         <v>10.69041667</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E18" s="18" t="n">
         <v>3335.41</v>
       </c>
-      <c r="F18" s="11" t="inlineStr">
+      <c r="F18" s="15" t="inlineStr">
         <is>
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/MOTOS</t>
         </is>
       </c>
-      <c r="G18" s="22" t="inlineStr">
+      <c r="G18" s="26" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="H18" s="18" t="n">
         <v>3230</v>
       </c>
-      <c r="I18" s="18" t="n">
+      <c r="I18" s="21" t="n">
         <v>-105.4099999999999</v>
       </c>
-      <c r="J18" s="27" t="n">
+      <c r="J18" s="31" t="n">
         <v>-0.03160331113716151</v>
       </c>
-      <c r="K18" s="11" t="inlineStr">
+      <c r="K18" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="L18" s="23" t="inlineStr">
+        <is>
+          <t>CPR $10.69 arriba del rango eficiente del producto. Bajar budget y mover el spend a los ad sets que mejor convierten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="50" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>MENSAJES_VIAJES_WHATSAPP_2025</t>
         </is>
       </c>
-      <c r="C19" s="24" t="n">
+      <c r="C19" s="28" t="n">
         <v>784</v>
       </c>
-      <c r="D19" s="14" t="n">
+      <c r="D19" s="16" t="n">
         <v>0.66506378</v>
       </c>
-      <c r="E19" s="5" t="n">
+      <c r="E19" s="18" t="n">
         <v>521.41</v>
       </c>
-      <c r="F19" s="11" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
         <is>
           <t>actions:onsite_conversion.messaging_conversation_started_7d</t>
         </is>
       </c>
-      <c r="G19" s="17" t="inlineStr">
+      <c r="G19" s="20" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE</t>
         </is>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="H19" s="18" t="n">
         <v>2068</v>
       </c>
-      <c r="I19" s="18" t="n">
+      <c r="I19" s="21" t="n">
         <v>1546.59</v>
       </c>
-      <c r="J19" s="25" t="n">
+      <c r="J19" s="29" t="n">
         <v>2.966168658061795</v>
       </c>
-      <c r="K19" s="11" t="inlineStr">
+      <c r="K19" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>CPR $0.67 excepcional (784 conversaciones WhatsApp). Es un outlier eficiente del MCC - vale la pena duplicar inversión y dejar que escale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_VIAJES_INTERESES_2025_V2</t>
         </is>
       </c>
-      <c r="C20" s="24" t="n">
+      <c r="C20" s="28" t="n">
         <v>41</v>
       </c>
-      <c r="D20" s="14" t="n">
+      <c r="D20" s="16" t="n">
         <v>28.6402439</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="18" t="n">
         <v>1174.25</v>
       </c>
-      <c r="F20" s="11" t="inlineStr">
+      <c r="F20" s="15" t="inlineStr">
         <is>
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G20" s="23" t="inlineStr">
+      <c r="G20" s="27" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE</t>
         </is>
       </c>
-      <c r="H20" s="5" t="n">
+      <c r="H20" s="18" t="n">
         <v>1035</v>
       </c>
-      <c r="I20" s="18" t="n">
+      <c r="I20" s="21" t="n">
         <v>-139.25</v>
       </c>
-      <c r="J20" s="27" t="n">
+      <c r="J20" s="31" t="n">
         <v>-0.1185863317010858</v>
       </c>
-      <c r="K20" s="11" t="inlineStr">
+      <c r="K20" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="L20" s="23" t="inlineStr">
+        <is>
+          <t>CPR $28.64 muy alto. $1,174 generaron solo 41 conversiones web. Pausar/recortar y reformular antes de seguir gastando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="50" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_VIAJES_RMKT_2025_V2</t>
         </is>
       </c>
-      <c r="C21" s="24" t="n">
+      <c r="C21" s="28" t="n">
         <v>37</v>
       </c>
-      <c r="D21" s="14" t="n">
+      <c r="D21" s="16" t="n">
         <v>31.48378378</v>
       </c>
-      <c r="E21" s="5" t="n">
+      <c r="E21" s="18" t="n">
         <v>1164.9</v>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G21" s="23" t="inlineStr">
+      <c r="G21" s="27" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE</t>
         </is>
       </c>
-      <c r="H21" s="5" t="n">
+      <c r="H21" s="18" t="n">
         <v>1027</v>
       </c>
-      <c r="I21" s="18" t="n">
+      <c r="I21" s="21" t="n">
         <v>-137.9000000000001</v>
       </c>
-      <c r="J21" s="27" t="n">
+      <c r="J21" s="31" t="n">
         <v>-0.1183792600223196</v>
       </c>
-      <c r="K21" s="11" t="inlineStr">
+      <c r="K21" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t>CPR $31.48 muy alto. $1,165 generaron solo 37 conversiones web. Pausar/recortar y reformular antes de seguir gastando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="50" customHeight="1">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_VIAJES_RMKT_PROMOCIONES</t>
         </is>
       </c>
-      <c r="C22" s="24" t="n">
+      <c r="C22" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="D22" s="14" t="n">
+      <c r="D22" s="16" t="n">
         <v>34.17285714</v>
       </c>
-      <c r="E22" s="5" t="n">
+      <c r="E22" s="18" t="n">
         <v>239.21</v>
       </c>
-      <c r="F22" s="11" t="inlineStr">
+      <c r="F22" s="15" t="inlineStr">
         <is>
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G22" s="23" t="inlineStr">
+      <c r="G22" s="27" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE</t>
         </is>
       </c>
-      <c r="H22" s="5" t="n">
+      <c r="H22" s="18" t="n">
         <v>211</v>
       </c>
-      <c r="I22" s="18" t="n">
+      <c r="I22" s="21" t="n">
         <v>-28.21000000000001</v>
       </c>
-      <c r="J22" s="27" t="n">
+      <c r="J22" s="31" t="n">
         <v>-0.1179298524309185</v>
       </c>
-      <c r="K22" s="11" t="inlineStr">
+      <c r="K22" s="15" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="L22" s="23" t="inlineStr">
+        <is>
+          <t>CPR $34.17 muy alto. $239 generaron solo 7 conversiones web. Pausar/recortar y reformular antes de seguir gastando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="50" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>CONVERSIONES_VIAJES_INTERESES_PROMOCIONES</t>
         </is>
       </c>
-      <c r="C23" s="24" t="n">
+      <c r="C23" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="D23" s="14" t="n">
+      <c r="D23" s="16" t="n">
         <v>48.606</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E23" s="18" t="n">
         <v>243.03</v>
       </c>
-      <c r="F23" s="11" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G23" s="23" t="inlineStr">
+      <c r="G23" s="27" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE</t>
         </is>
       </c>
-      <c r="H23" s="5" t="n">
+      <c r="H23" s="18" t="n">
         <v>214</v>
       </c>
-      <c r="I23" s="18" t="n">
+      <c r="I23" s="21" t="n">
         <v>-29.03</v>
       </c>
-      <c r="J23" s="27" t="n">
+      <c r="J23" s="31" t="n">
         <v>-0.1194502736287701</v>
       </c>
-      <c r="K23" s="11" t="inlineStr">
+      <c r="K23" s="15" t="inlineStr">
         <is>
           <t>active</t>
+        </is>
+      </c>
+      <c r="L23" s="23" t="inlineStr">
+        <is>
+          <t>CPR $48.61 muy alto. $243 generaron solo 5 conversiones web. Pausar/recortar y reformular antes de seguir gastando.</t>
         </is>
       </c>
     </row>
@@ -2647,22 +2867,22 @@
           <t>Auto</t>
         </is>
       </c>
-      <c r="B28" s="28" t="n">
+      <c r="B28" s="32" t="n">
         <v>6</v>
       </c>
       <c r="C28" s="5" t="n">
         <v>10625.42</v>
       </c>
-      <c r="D28" s="24" t="n">
+      <c r="D28" s="33" t="n">
         <v>2619</v>
       </c>
-      <c r="E28" s="14" t="n">
+      <c r="E28" s="34" t="n">
         <v>4.057052310042</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>13558</v>
       </c>
-      <c r="G28" s="18" t="n">
+      <c r="G28" s="35" t="n">
         <v>2932.580000000002</v>
       </c>
     </row>
@@ -2672,22 +2892,22 @@
           <t>Moto</t>
         </is>
       </c>
-      <c r="B29" s="28" t="n">
+      <c r="B29" s="32" t="n">
         <v>3</v>
       </c>
       <c r="C29" s="5" t="n">
         <v>6948.599999999999</v>
       </c>
-      <c r="D29" s="24" t="n">
+      <c r="D29" s="33" t="n">
         <v>1237</v>
       </c>
-      <c r="E29" s="14" t="n">
+      <c r="E29" s="34" t="n">
         <v>5.617299919159255</v>
       </c>
       <c r="F29" s="5" t="n">
         <v>8387</v>
       </c>
-      <c r="G29" s="18" t="n">
+      <c r="G29" s="35" t="n">
         <v>1438.400000000001</v>
       </c>
     </row>
@@ -2697,22 +2917,22 @@
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="B30" s="28" t="n">
+      <c r="B30" s="32" t="n">
         <v>5</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>8513.869999999999</v>
       </c>
-      <c r="D30" s="24" t="n">
+      <c r="D30" s="33" t="n">
         <v>2217</v>
       </c>
-      <c r="E30" s="14" t="n">
+      <c r="E30" s="34" t="n">
         <v>3.840266125394677</v>
       </c>
       <c r="F30" s="5" t="n">
         <v>7535</v>
       </c>
-      <c r="G30" s="18" t="n">
+      <c r="G30" s="35" t="n">
         <v>-978.869999999999</v>
       </c>
     </row>
@@ -2722,22 +2942,22 @@
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B31" s="28" t="n">
+      <c r="B31" s="32" t="n">
         <v>5</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>3342.8</v>
       </c>
-      <c r="D31" s="24" t="n">
+      <c r="D31" s="33" t="n">
         <v>874</v>
       </c>
-      <c r="E31" s="14" t="n">
+      <c r="E31" s="34" t="n">
         <v>3.824713958810069</v>
       </c>
       <c r="F31" s="5" t="n">
         <v>4555</v>
       </c>
-      <c r="G31" s="18" t="n">
+      <c r="G31" s="35" t="n">
         <v>1212.2</v>
       </c>
     </row>
@@ -2771,208 +2991,208 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="29" t="inlineStr">
+      <c r="A3" s="36" t="inlineStr">
         <is>
           <t>Datos base</t>
         </is>
       </c>
-      <c r="B3" s="30" t="inlineStr">
+      <c r="B3" s="37" t="inlineStr">
         <is>
           <t>Performance real del 1-27 abril 2026 cruzado con Sheet Leads CRM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="36" t="inlineStr">
         <is>
           <t>Constraint 1</t>
         </is>
       </c>
-      <c r="B4" s="30" t="inlineStr">
+      <c r="B4" s="37" t="inlineStr">
         <is>
           <t>Tope por seguro provisto por el cliente (Auto $52.421, Moto $32.642, Arriendo $31.080, Viajes $16.900)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t>Constraint 2</t>
         </is>
       </c>
-      <c r="B5" s="30" t="inlineStr">
+      <c r="B5" s="37" t="inlineStr">
         <is>
           <t>70-75% del presupuesto en Google (mejor calidad de leads SF según cliente)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="36" t="inlineStr">
         <is>
           <t>Constraint 3</t>
         </is>
       </c>
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="37" t="inlineStr">
         <is>
           <t>Bing se mantiene en presupuesto del Flow</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="31" t="inlineStr"/>
-      <c r="B7" s="30" t="inlineStr"/>
+      <c r="A7" s="38" t="inlineStr"/>
+      <c r="B7" s="37" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="32" t="inlineStr">
+      <c r="A8" s="39" t="inlineStr">
         <is>
           <t>Reglas de clasificación de campañas Google</t>
         </is>
       </c>
-      <c r="B8" s="30" t="inlineStr"/>
+      <c r="B8" s="37" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE (×1.80)</t>
         </is>
       </c>
-      <c r="B9" s="30" t="inlineStr">
+      <c r="B9" s="37" t="inlineStr">
         <is>
           <t>CPA ≤ $7 y % Lost Budget ≥ 50% — palanca #1</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="36" t="inlineStr">
         <is>
           <t>ESCALAR (×1.40)</t>
         </is>
       </c>
-      <c r="B10" s="30" t="inlineStr">
+      <c r="B10" s="37" t="inlineStr">
         <is>
           <t>CPA ≤ $10 y % Lost Budget ≥ 30%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="36" t="inlineStr">
         <is>
           <t>ESCALAR LEVE (×1.20)</t>
         </is>
       </c>
-      <c r="B11" s="30" t="inlineStr">
+      <c r="B11" s="37" t="inlineStr">
         <is>
           <t>CPA ≤ $10 y % Lost Budget ≥ 10%</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="36" t="inlineStr">
         <is>
           <t>ESCALAR MODERADO (×1.20)</t>
         </is>
       </c>
-      <c r="B12" s="30" t="inlineStr">
+      <c r="B12" s="37" t="inlineStr">
         <is>
           <t>CPA ≤ $15 y % Lost Budget ≥ 50%</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="36" t="inlineStr">
         <is>
           <t>RECORTAR (×0.65)</t>
         </is>
       </c>
-      <c r="B13" s="30" t="inlineStr">
+      <c r="B13" s="37" t="inlineStr">
         <is>
           <t>CPA entre $15 y $25</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="36" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE (×0.40)</t>
         </is>
       </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="37" t="inlineStr">
         <is>
           <t>CPA &gt; $25</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="36" t="inlineStr">
         <is>
           <t>MANTENER (×1.00)</t>
         </is>
       </c>
-      <c r="B15" s="30" t="inlineStr">
+      <c r="B15" s="37" t="inlineStr">
         <is>
           <t>Resto</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr"/>
-      <c r="B16" s="30" t="inlineStr"/>
+      <c r="A16" s="38" t="inlineStr"/>
+      <c r="B16" s="37" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A17" s="36" t="inlineStr">
         <is>
           <t>Ajuste fino</t>
         </is>
       </c>
-      <c r="B17" s="30" t="inlineStr">
+      <c r="B17" s="37" t="inlineStr">
         <is>
           <t>Después del factor inicial, los presupuestos de Google se reescalan proporcionalmente para alcanzar exactamente el 72% del total por seguro.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="31" t="inlineStr"/>
-      <c r="B18" s="30" t="inlineStr"/>
+      <c r="A18" s="38" t="inlineStr"/>
+      <c r="B18" s="37" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="A19" s="39" t="inlineStr">
         <is>
           <t>Limitaciones honestas</t>
         </is>
       </c>
-      <c r="B19" s="30" t="inlineStr"/>
+      <c r="B19" s="37" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="36" t="inlineStr">
         <is>
           <t>Meta</t>
         </is>
       </c>
-      <c r="B20" s="30" t="inlineStr">
+      <c r="B20" s="37" t="inlineStr">
         <is>
           <t>Detalle por ad set requiere CSV exportado del Ads Manager (Reports → Export Reports). Esta propuesta optimiza Meta a nivel seguro.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="29" t="inlineStr">
+      <c r="A21" s="36" t="inlineStr">
         <is>
           <t>Bing</t>
         </is>
       </c>
-      <c r="B21" s="30" t="inlineStr">
+      <c r="B21" s="37" t="inlineStr">
         <is>
           <t>No se modificó (sin acceso desde el extractor).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="29" t="inlineStr">
+      <c r="A22" s="36" t="inlineStr">
         <is>
           <t>Estacionalidad</t>
         </is>
       </c>
-      <c r="B22" s="30" t="inlineStr">
+      <c r="B22" s="37" t="inlineStr">
         <is>
           <t>Asume ritmo similar a abril. Si hay cambios estacionales, ajustar.</t>
         </is>

</xml_diff>

<commit_message>
feat(dev): tasa de conversion incorporada en clasificador y justificacion Google
Cambios:
- Cargo campanias Google del dataset real (data_paid_media.json) en lugar de
  hardcoded - esto trae clicks y permite calcular tasa_conv = conv/clicks
- Funcion clasificar() ahora considera 3 variables:
    * CPA
    * % Lost Budget
    * Tasa de conversion (alta >=8% / media 4-8% / baja <4%)
- ESCALAR FUERTE solo se aplica si tasa de conversion es alta o media
- Si CPA medio-alto con tasa baja -> RECORTAR (problema de funnel)
- Hoja 'Detalle Google' tiene nueva columna 'Tasa conv.' (verde si >=8%, rojo si <4%)
- Justificacion ahora incluye explicitamente la tasa de conversion como parte
  del razonamiento ('CPA $X + tasa conv Y% (eval)')

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/suratech_propuesta_distribucion_mayo2026.xlsx
+++ b/outputs/suratech_propuesta_distribucion_mayo2026.xlsx
@@ -127,12 +127,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
+        <fgColor rgb="00ECFDF5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ECFDF5"/>
+        <fgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
     <fill>
@@ -172,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -198,10 +198,16 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -219,19 +225,19 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="169" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -706,10 +712,10 @@
         <v>26132</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>37742</v>
+        <v>37743</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>11610</v>
+        <v>11611</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>10244</v>
@@ -737,10 +743,10 @@
         <v>15555</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>23503</v>
+        <v>23502</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>7948</v>
+        <v>7947</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>6629</v>
@@ -768,10 +774,10 @@
         <v>28902</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>22378</v>
+        <v>22379</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>-6524</v>
+        <v>-6523</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>8083</v>
@@ -830,10 +836,10 @@
         <v>77351</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>95791</v>
+        <v>95792</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>18440</v>
+        <v>18441</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>28142</v>
@@ -1030,21 +1036,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="70" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="75" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1072,51 +1080,61 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>Tasa conv.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
           <t>% Lost Budget</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Budget/día actual</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Spend actual</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Conversiones actuales</t>
-        </is>
-      </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Conversiones</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
           <t>Acción</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Spend propuesto</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Δ Spend</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Δ %</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Justificación</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="50" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Auto</t>
@@ -1124,367 +1142,415 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
+          <t>SURA_AUTOS_SEARCH_SEGMENT</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>0.1645948545323395</v>
+      </c>
+      <c r="E4" s="18" t="n">
+        <v>0.1459</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>326</v>
+      </c>
+      <c r="G4" s="19" t="n">
+        <v>9197.959999999999</v>
+      </c>
+      <c r="H4" s="20" t="n">
+        <v>8318</v>
+      </c>
+      <c r="I4" s="21" t="n">
+        <v>1369.1</v>
+      </c>
+      <c r="J4" s="22" t="inlineStr">
+        <is>
+          <t>ESCALAR LEVE</t>
+        </is>
+      </c>
+      <c r="K4" s="19" t="n">
+        <v>11108</v>
+      </c>
+      <c r="L4" s="23" t="n">
+        <v>1910.040000000001</v>
+      </c>
+      <c r="M4" s="24" t="n">
+        <v>0.2076590896242211</v>
+      </c>
+      <c r="N4" s="25" t="inlineStr">
+        <is>
+          <t>CPA $6.72, tasa conv 16.5% (alta), 1,369 conversiones validan el formato, 15% lost budget = headroom. Subir budget para capitalizar la eficiencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>SURA_AUTOS_SEARCH_RETENTION</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>0.1350630753494715</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>0.2289</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>147</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>4194</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <v>2933</v>
+      </c>
+      <c r="I5" s="21" t="n">
+        <v>396.14</v>
+      </c>
+      <c r="J5" s="26" t="inlineStr">
+        <is>
+          <t>MANTENER</t>
+        </is>
+      </c>
+      <c r="K5" s="19" t="n">
+        <v>4221</v>
+      </c>
+      <c r="L5" s="23" t="n">
+        <v>27</v>
+      </c>
+      <c r="M5" s="24" t="n">
+        <v>0.006437768240343348</v>
+      </c>
+      <c r="N5" s="25" t="inlineStr">
+        <is>
+          <t>CPA $10.59, tasa conv 13.5%. Monitorear y mantener estable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>SURA_AUTOS_SEARCH_CONQUEST</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>0.163258480649785</v>
+      </c>
+      <c r="E6" s="18" t="n">
+        <v>0.4165</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>52</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>2188.75</v>
+      </c>
+      <c r="H6" s="20" t="n">
+        <v>2093</v>
+      </c>
+      <c r="I6" s="21" t="n">
+        <v>341.7</v>
+      </c>
+      <c r="J6" s="22" t="inlineStr">
+        <is>
+          <t>ESCALAR</t>
+        </is>
+      </c>
+      <c r="K6" s="19" t="n">
+        <v>3083</v>
+      </c>
+      <c r="L6" s="23" t="n">
+        <v>894.25</v>
+      </c>
+      <c r="M6" s="24" t="n">
+        <v>0.4085665334094803</v>
+      </c>
+      <c r="N6" s="25" t="inlineStr">
+        <is>
+          <t>CPA $6.41, tasa conv 16.3% (alta), 341 conversiones validan el formato, 42% lost budget = headroom. Subir budget para capitalizar la eficiencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
           <t>SURA_AUTOS_PMAX</t>
         </is>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="C7" s="16" t="n">
         <v>3.9</v>
       </c>
-      <c r="D4" s="17" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="E4" s="18" t="n">
+      <c r="D7" s="17" t="n">
+        <v>0.1840155840666353</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>0.7423999999999999</v>
+      </c>
+      <c r="F7" s="19" t="n">
         <v>517</v>
       </c>
-      <c r="F4" s="18" t="n">
-        <v>10672</v>
-      </c>
-      <c r="G4" s="19" t="n">
-        <v>2739.4</v>
-      </c>
-      <c r="H4" s="20" t="inlineStr">
+      <c r="G7" s="19" t="n">
+        <v>10671.99</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <v>14887</v>
+      </c>
+      <c r="I7" s="21" t="n">
+        <v>2739.44</v>
+      </c>
+      <c r="J7" s="27" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE</t>
         </is>
       </c>
-      <c r="I4" s="18" t="n">
+      <c r="K7" s="19" t="n">
         <v>19331</v>
       </c>
-      <c r="J4" s="21" t="n">
-        <v>8659</v>
-      </c>
-      <c r="K4" s="22" t="n">
-        <v>0.8113755622188905</v>
-      </c>
-      <c r="L4" s="23" t="inlineStr">
-        <is>
-          <t>CPA $3.90 excelente y pierde 74% de impresiones por presupuesto. Subir budget convierte impresiones perdidas en conversiones al mismo CPA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="50" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>SURA_AUTOS_SEARCH_SEGMENT</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="n">
-        <v>6.72</v>
-      </c>
-      <c r="D5" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E5" s="18" t="n">
-        <v>326</v>
-      </c>
-      <c r="F5" s="18" t="n">
-        <v>9198</v>
-      </c>
-      <c r="G5" s="19" t="n">
-        <v>1369.1</v>
-      </c>
-      <c r="H5" s="24" t="inlineStr">
-        <is>
-          <t>ESCALAR LEVE</t>
-        </is>
-      </c>
-      <c r="I5" s="18" t="n">
-        <v>11107</v>
-      </c>
-      <c r="J5" s="21" t="n">
-        <v>1909</v>
-      </c>
-      <c r="K5" s="22" t="n">
-        <v>0.2075451185040226</v>
-      </c>
-      <c r="L5" s="23" t="inlineStr">
-        <is>
-          <t>CPA $6.72, 1,369 conversiones ya validan el formato, 15% lost budget = headroom. Subir budget para capitalizar la eficiencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="50" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>SURA_AUTOS_SEARCH_RETENTION</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="n">
-        <v>10.59</v>
-      </c>
-      <c r="D6" s="17" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="E6" s="18" t="n">
-        <v>147</v>
-      </c>
-      <c r="F6" s="18" t="n">
-        <v>4194</v>
-      </c>
-      <c r="G6" s="19" t="n">
-        <v>396.1</v>
-      </c>
-      <c r="H6" s="25" t="inlineStr">
+      <c r="L7" s="23" t="n">
+        <v>8659.01</v>
+      </c>
+      <c r="M7" s="24" t="n">
+        <v>0.8113772595364126</v>
+      </c>
+      <c r="N7" s="25" t="inlineStr">
+        <is>
+          <t>CPA $3.90 + tasa de conversión 18.4% (alta) + pierde 74% por presupuesto. Combo ideal: convierte bien y le falta plata. Subir budget convierte impresiones perdidas en conversiones al mismo CPA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Moto</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>SURA_MOTOS_SEARCH_SEGMENT</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="D9" s="28" t="n">
+        <v>0.03343319284656567</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>0.6555</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>357</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>4595.78</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>8779</v>
+      </c>
+      <c r="I9" s="21" t="n">
+        <v>293.51</v>
+      </c>
+      <c r="J9" s="29" t="inlineStr">
+        <is>
+          <t>RECORTAR</t>
+        </is>
+      </c>
+      <c r="K9" s="19" t="n">
+        <v>6137</v>
+      </c>
+      <c r="L9" s="23" t="n">
+        <v>1541.22</v>
+      </c>
+      <c r="M9" s="24" t="n">
+        <v>0.3353554782866021</v>
+      </c>
+      <c r="N9" s="25" t="inlineStr">
+        <is>
+          <t>Tasa de conversión 3.3% (baja) sobre 8,779 clicks → el funnel no convierte bien. CPA $15.66. Recortar y revisar landing/oferta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Moto</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>SURA_MOTOS_SEARCH_RETENTION</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>0.07868535031847133</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>0.0384</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>183</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>1993.64</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <v>3925</v>
+      </c>
+      <c r="I10" s="21" t="n">
+        <v>308.84</v>
+      </c>
+      <c r="J10" s="26" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="I6" s="18" t="n">
-        <v>4220</v>
-      </c>
-      <c r="J6" s="21" t="n">
-        <v>26</v>
-      </c>
-      <c r="K6" s="22" t="n">
-        <v>0.00619933237958989</v>
-      </c>
-      <c r="L6" s="23" t="inlineStr">
-        <is>
-          <t>CPA $10.59. Monitorear y mantener estable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="50" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
-        <is>
-          <t>SURA_AUTOS_SEARCH_CONQUEST</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="n">
-        <v>6.41</v>
-      </c>
-      <c r="D7" s="17" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="E7" s="18" t="n">
-        <v>52</v>
-      </c>
-      <c r="F7" s="18" t="n">
-        <v>2189</v>
-      </c>
-      <c r="G7" s="19" t="n">
-        <v>341.7</v>
-      </c>
-      <c r="H7" s="24" t="inlineStr">
-        <is>
-          <t>ESCALAR</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="n">
-        <v>3084</v>
-      </c>
-      <c r="J7" s="21" t="n">
-        <v>895</v>
-      </c>
-      <c r="K7" s="22" t="n">
-        <v>0.40886249428963</v>
-      </c>
-      <c r="L7" s="23" t="inlineStr">
-        <is>
-          <t>CPA $6.41, 341 conversiones ya validan el formato, 42% lost budget = headroom. Subir budget para capitalizar la eficiencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="50" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="K10" s="19" t="n">
+        <v>4097</v>
+      </c>
+      <c r="L10" s="23" t="n">
+        <v>2103.36</v>
+      </c>
+      <c r="M10" s="24" t="n">
+        <v>1.055035011336048</v>
+      </c>
+      <c r="N10" s="25" t="inlineStr">
+        <is>
+          <t>CPA $6.46 + tasa conv 7.9% aceptables, la campaña ya consume su budget (lost 4%). Sin headroom para escalar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Moto</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>SURA_MOTOS_SEARCH_RETENTION</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>6.46</v>
-      </c>
-      <c r="D9" s="17" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="E9" s="18" t="n">
-        <v>183</v>
-      </c>
-      <c r="F9" s="18" t="n">
-        <v>1994</v>
-      </c>
-      <c r="G9" s="19" t="n">
-        <v>308.8</v>
-      </c>
-      <c r="H9" s="25" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>SURA_MOTOS_SEARCH_CONQUEST</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>0.04215982721382289</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>0.7295999999999999</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>75</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>1366.13</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <v>2315</v>
+      </c>
+      <c r="I11" s="21" t="n">
+        <v>97.59999999999999</v>
+      </c>
+      <c r="J11" s="26" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="I9" s="18" t="n">
-        <v>2926</v>
-      </c>
-      <c r="J9" s="21" t="n">
-        <v>932</v>
-      </c>
-      <c r="K9" s="22" t="n">
-        <v>0.4674022066198596</v>
-      </c>
-      <c r="L9" s="23" t="inlineStr">
-        <is>
-          <t>CPA $6.46 aceptable y la campaña ya consume su budget (lost 4%). Sin headroom para escalar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="50" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="K11" s="19" t="n">
+        <v>2807</v>
+      </c>
+      <c r="L11" s="23" t="n">
+        <v>1440.87</v>
+      </c>
+      <c r="M11" s="24" t="n">
+        <v>1.054709288281496</v>
+      </c>
+      <c r="N11" s="25" t="inlineStr">
+        <is>
+          <t>CPA $14.00, tasa conv 4.2%. Monitorear y mantener estable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Moto</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>SURA_MOTOS_PMAX</t>
         </is>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C12" s="16" t="n">
         <v>12.19</v>
       </c>
-      <c r="D10" s="17" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E10" s="18" t="n">
+      <c r="D12" s="28" t="n">
+        <v>0.002189902142506678</v>
+      </c>
+      <c r="E12" s="18" t="n">
+        <v>0.5758</v>
+      </c>
+      <c r="F12" s="19" t="n">
         <v>397</v>
       </c>
-      <c r="F10" s="18" t="n">
-        <v>7832</v>
-      </c>
-      <c r="G10" s="19" t="n">
-        <v>642.7</v>
-      </c>
-      <c r="H10" s="24" t="inlineStr">
-        <is>
-          <t>ESCALAR MODERADO</t>
-        </is>
-      </c>
-      <c r="I10" s="18" t="n">
-        <v>13789</v>
-      </c>
-      <c r="J10" s="21" t="n">
-        <v>5957</v>
-      </c>
-      <c r="K10" s="22" t="n">
-        <v>0.7605975485188968</v>
-      </c>
-      <c r="L10" s="23" t="inlineStr">
-        <is>
-          <t>CPA $12.19, 642 conversiones ya validan el formato, 58% lost budget = headroom. Subir budget para capitalizar la eficiencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="50" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>Moto</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="inlineStr">
-        <is>
-          <t>SURA_MOTOS_SEARCH_SEGMENT</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="n">
-        <v>15.66</v>
-      </c>
-      <c r="D11" s="17" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="E11" s="18" t="n">
-        <v>357</v>
-      </c>
-      <c r="F11" s="18" t="n">
-        <v>4596</v>
-      </c>
-      <c r="G11" s="19" t="n">
-        <v>293.5</v>
-      </c>
-      <c r="H11" s="26" t="inlineStr">
+      <c r="G12" s="19" t="n">
+        <v>7831.97</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <v>293488</v>
+      </c>
+      <c r="I12" s="21" t="n">
+        <v>642.71</v>
+      </c>
+      <c r="J12" s="29" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="I11" s="18" t="n">
-        <v>4383</v>
-      </c>
-      <c r="J11" s="21" t="n">
-        <v>-213</v>
-      </c>
-      <c r="K11" s="22" t="n">
-        <v>-0.04634464751958225</v>
-      </c>
-      <c r="L11" s="23" t="inlineStr">
-        <is>
-          <t>CPA $15.66 alto + tiene anuncios rechazados. Recortar mientras se corrigen los assets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="50" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>Moto</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>SURA_MOTOS_SEARCH_CONQUEST</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="n">
-        <v>14</v>
-      </c>
-      <c r="D12" s="17" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="E12" s="18" t="n">
-        <v>75</v>
-      </c>
-      <c r="F12" s="18" t="n">
-        <v>1366</v>
-      </c>
-      <c r="G12" s="19" t="n">
-        <v>97.59999999999999</v>
-      </c>
-      <c r="H12" s="24" t="inlineStr">
-        <is>
-          <t>ESCALAR MODERADO</t>
-        </is>
-      </c>
-      <c r="I12" s="18" t="n">
-        <v>2405</v>
-      </c>
-      <c r="J12" s="21" t="n">
-        <v>1039</v>
-      </c>
-      <c r="K12" s="22" t="n">
-        <v>0.760614934114202</v>
-      </c>
-      <c r="L12" s="23" t="inlineStr">
-        <is>
-          <t>CPA $14.00, 73% lost budget = headroom. Subir budget para capitalizar la eficiencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="50" customHeight="1">
+      <c r="K12" s="19" t="n">
+        <v>10461</v>
+      </c>
+      <c r="L12" s="23" t="n">
+        <v>2629.03</v>
+      </c>
+      <c r="M12" s="24" t="n">
+        <v>0.3356792735416503</v>
+      </c>
+      <c r="N12" s="25" t="inlineStr">
+        <is>
+          <t>Tasa de conversión 0.2% (baja) sobre 293,488 clicks → el funnel no convierte bien. CPA $12.19. Recortar y revisar landing/oferta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Arriendo</t>
@@ -1499,38 +1565,44 @@
         <v>7.32</v>
       </c>
       <c r="D14" s="17" t="n">
-        <v>0.06</v>
+        <v>0.09964401485236046</v>
       </c>
       <c r="E14" s="18" t="n">
+        <v>0.0579</v>
+      </c>
+      <c r="F14" s="19" t="n">
         <v>984</v>
       </c>
-      <c r="F14" s="18" t="n">
-        <v>12383</v>
-      </c>
       <c r="G14" s="19" t="n">
-        <v>1690.7</v>
-      </c>
-      <c r="H14" s="25" t="inlineStr">
+        <v>12383.3</v>
+      </c>
+      <c r="H14" s="20" t="n">
+        <v>16967</v>
+      </c>
+      <c r="I14" s="21" t="n">
+        <v>1690.66</v>
+      </c>
+      <c r="J14" s="26" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="I14" s="18" t="n">
-        <v>13603</v>
-      </c>
-      <c r="J14" s="21" t="n">
-        <v>1220</v>
-      </c>
-      <c r="K14" s="22" t="n">
-        <v>0.09852216748768473</v>
-      </c>
-      <c r="L14" s="23" t="inlineStr">
-        <is>
-          <t>CPA $7.32 aceptable y la campaña ya consume su budget (lost 6%). Sin headroom para escalar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="50" customHeight="1">
+      <c r="K14" s="19" t="n">
+        <v>13604</v>
+      </c>
+      <c r="L14" s="23" t="n">
+        <v>1220.700000000001</v>
+      </c>
+      <c r="M14" s="24" t="n">
+        <v>0.09857630841536592</v>
+      </c>
+      <c r="N14" s="25" t="inlineStr">
+        <is>
+          <t>CPA $7.32 + tasa conv 10.0% aceptables, la campaña ya consume su budget (lost 6%). Sin headroom para escalar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Arriendo</t>
@@ -1544,39 +1616,45 @@
       <c r="C15" s="16" t="n">
         <v>25.27</v>
       </c>
-      <c r="D15" s="17" t="n">
-        <v>0.14</v>
+      <c r="D15" s="18" t="n">
+        <v>0.05069934436465813</v>
       </c>
       <c r="E15" s="18" t="n">
+        <v>0.1399</v>
+      </c>
+      <c r="F15" s="19" t="n">
         <v>900</v>
       </c>
-      <c r="F15" s="18" t="n">
-        <v>8208</v>
-      </c>
       <c r="G15" s="19" t="n">
-        <v>324.8</v>
-      </c>
-      <c r="H15" s="27" t="inlineStr">
+        <v>8208.290000000001</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <v>6406</v>
+      </c>
+      <c r="I15" s="21" t="n">
+        <v>324.78</v>
+      </c>
+      <c r="J15" s="30" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE</t>
         </is>
       </c>
-      <c r="I15" s="18" t="n">
-        <v>3606</v>
-      </c>
-      <c r="J15" s="21" t="n">
-        <v>-4602</v>
-      </c>
-      <c r="K15" s="22" t="n">
-        <v>-0.560672514619883</v>
-      </c>
-      <c r="L15" s="23" t="inlineStr">
-        <is>
-          <t>CPA $25.27 insostenible. $8,208 invertidos generaron solo 324 conversiones. Bajar budget y revisar keywords/creatividades antes de seguir gastando.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="50" customHeight="1">
+      <c r="K15" s="19" t="n">
+        <v>3607</v>
+      </c>
+      <c r="L15" s="23" t="n">
+        <v>-4601.290000000001</v>
+      </c>
+      <c r="M15" s="24" t="n">
+        <v>-0.5605662080652609</v>
+      </c>
+      <c r="N15" s="25" t="inlineStr">
+        <is>
+          <t>CPA $25.27 insostenible. Tasa conv 5.1% (media) sobre 6,406 clicks. $8,208 invertidos generaron solo 324 conversiones. Bajar budget y revisar keywords/landing antes de seguir gastando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Arriendo</t>
@@ -1590,39 +1668,45 @@
       <c r="C16" s="16" t="n">
         <v>23.55</v>
       </c>
-      <c r="D16" s="17" t="n">
-        <v>0.73</v>
+      <c r="D16" s="28" t="n">
+        <v>0.005403238567434991</v>
       </c>
       <c r="E16" s="18" t="n">
+        <v>0.7286</v>
+      </c>
+      <c r="F16" s="19" t="n">
         <v>376</v>
       </c>
-      <c r="F16" s="18" t="n">
-        <v>7238</v>
-      </c>
       <c r="G16" s="19" t="n">
-        <v>307.3</v>
-      </c>
-      <c r="H16" s="26" t="inlineStr">
+        <v>7237.62</v>
+      </c>
+      <c r="H16" s="20" t="n">
+        <v>56877</v>
+      </c>
+      <c r="I16" s="21" t="n">
+        <v>307.32</v>
+      </c>
+      <c r="J16" s="29" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="I16" s="18" t="n">
-        <v>5169</v>
-      </c>
-      <c r="J16" s="21" t="n">
-        <v>-2069</v>
-      </c>
-      <c r="K16" s="22" t="n">
-        <v>-0.2858524454269135</v>
-      </c>
-      <c r="L16" s="23" t="inlineStr">
-        <is>
-          <t>CPA $23.55 fuera de rango. Recortar y mover budget a campañas más eficientes del seguro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="50" customHeight="1">
+      <c r="K16" s="19" t="n">
+        <v>5168</v>
+      </c>
+      <c r="L16" s="23" t="n">
+        <v>-2069.62</v>
+      </c>
+      <c r="M16" s="24" t="n">
+        <v>-0.2859531171849309</v>
+      </c>
+      <c r="N16" s="25" t="inlineStr">
+        <is>
+          <t>Tasa de conversión 0.5% (baja) sobre 56,877 clicks → el funnel no convierte bien. CPA $23.55. Recortar y revisar landing/oferta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Viajes</t>
@@ -1630,139 +1714,157 @@
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
+          <t>SURA_VIAJES_SEARCH_SEGMENT</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>54.52</v>
+      </c>
+      <c r="D18" s="28" t="n">
+        <v>0.02732997481108312</v>
+      </c>
+      <c r="E18" s="18" t="n">
+        <v>0.5768</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>106</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>1774.72</v>
+      </c>
+      <c r="H18" s="20" t="n">
+        <v>1191</v>
+      </c>
+      <c r="I18" s="21" t="n">
+        <v>32.55</v>
+      </c>
+      <c r="J18" s="30" t="inlineStr">
+        <is>
+          <t>RECORTAR FUERTE</t>
+        </is>
+      </c>
+      <c r="K18" s="19" t="n">
+        <v>2207</v>
+      </c>
+      <c r="L18" s="23" t="n">
+        <v>432.28</v>
+      </c>
+      <c r="M18" s="24" t="n">
+        <v>0.2435764514965741</v>
+      </c>
+      <c r="N18" s="25" t="inlineStr">
+        <is>
+          <t>CPA $54.52 insostenible. Tasa conv 2.7% (baja) sobre 1,191 clicks. $1,775 invertidos generaron solo 32 conversiones. Bajar budget y revisar keywords/landing antes de seguir gastando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
           <t>SURA_VIAJES_SEARCH_RETENTION</t>
         </is>
       </c>
-      <c r="C18" s="16" t="n">
+      <c r="C19" s="16" t="n">
         <v>22.67</v>
       </c>
-      <c r="D18" s="17" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E18" s="18" t="n">
+      <c r="D19" s="18" t="n">
+        <v>0.05792661361626879</v>
+      </c>
+      <c r="E19" s="18" t="n">
+        <v>0.201</v>
+      </c>
+      <c r="F19" s="19" t="n">
         <v>251</v>
       </c>
-      <c r="F18" s="18" t="n">
-        <v>2971</v>
-      </c>
-      <c r="G18" s="19" t="n">
-        <v>131</v>
-      </c>
-      <c r="H18" s="26" t="inlineStr">
+      <c r="G19" s="19" t="n">
+        <v>2970.71</v>
+      </c>
+      <c r="H19" s="20" t="n">
+        <v>2262</v>
+      </c>
+      <c r="I19" s="21" t="n">
+        <v>131.03</v>
+      </c>
+      <c r="J19" s="29" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="I18" s="18" t="n">
+      <c r="K19" s="19" t="n">
         <v>6003</v>
       </c>
-      <c r="J18" s="21" t="n">
-        <v>3032</v>
-      </c>
-      <c r="K18" s="22" t="n">
-        <v>1.020531807472232</v>
-      </c>
-      <c r="L18" s="23" t="inlineStr">
-        <is>
-          <t>CPA $22.67 fuera de rango. Recortar y mover budget a campañas más eficientes del seguro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="50" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="L19" s="23" t="n">
+        <v>3032.29</v>
+      </c>
+      <c r="M19" s="24" t="n">
+        <v>1.020729051304234</v>
+      </c>
+      <c r="N19" s="25" t="inlineStr">
+        <is>
+          <t>CPA $22.67 fuera de rango con tasa conv 5.8%. Recortar y mover budget a campañas más eficientes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>SURA_VIAJES_PMAX</t>
         </is>
       </c>
-      <c r="C19" s="16" t="n">
+      <c r="C20" s="16" t="n">
         <v>20.66</v>
       </c>
-      <c r="D19" s="17" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="E19" s="18" t="n">
+      <c r="D20" s="28" t="n">
+        <v>0.01390029325513197</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>0.7689</v>
+      </c>
+      <c r="F20" s="19" t="n">
         <v>155</v>
       </c>
-      <c r="F19" s="18" t="n">
-        <v>1959</v>
-      </c>
-      <c r="G19" s="19" t="n">
+      <c r="G20" s="19" t="n">
+        <v>1958.93</v>
+      </c>
+      <c r="H20" s="20" t="n">
+        <v>6820</v>
+      </c>
+      <c r="I20" s="21" t="n">
         <v>94.8</v>
       </c>
-      <c r="H19" s="26" t="inlineStr">
+      <c r="J20" s="29" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="I19" s="18" t="n">
+      <c r="K20" s="19" t="n">
         <v>3958</v>
       </c>
-      <c r="J19" s="21" t="n">
-        <v>1999</v>
-      </c>
-      <c r="K19" s="22" t="n">
-        <v>1.020418580908627</v>
-      </c>
-      <c r="L19" s="23" t="inlineStr">
-        <is>
-          <t>CPA $20.66 fuera de rango. Recortar y mover budget a campañas más eficientes del seguro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="50" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>Viajes</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>SURA_VIAJES_SEARCH_SEGMENT</t>
-        </is>
-      </c>
-      <c r="C20" s="16" t="n">
-        <v>54.52</v>
-      </c>
-      <c r="D20" s="17" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="E20" s="18" t="n">
-        <v>106</v>
-      </c>
-      <c r="F20" s="18" t="n">
-        <v>1775</v>
-      </c>
-      <c r="G20" s="19" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="H20" s="27" t="inlineStr">
-        <is>
-          <t>RECORTAR FUERTE</t>
-        </is>
-      </c>
-      <c r="I20" s="18" t="n">
-        <v>2207</v>
-      </c>
-      <c r="J20" s="21" t="n">
-        <v>432</v>
-      </c>
-      <c r="K20" s="22" t="n">
-        <v>0.2433802816901408</v>
-      </c>
-      <c r="L20" s="23" t="inlineStr">
-        <is>
-          <t>CPA $54.52 insostenible. $1,775 invertidos generaron solo 32 conversiones. Bajar budget y revisar keywords/creatividades antes de seguir gastando.</t>
+      <c r="L20" s="23" t="n">
+        <v>1999.07</v>
+      </c>
+      <c r="M20" s="24" t="n">
+        <v>1.020490778128876</v>
+      </c>
+      <c r="N20" s="25" t="inlineStr">
+        <is>
+          <t>Tasa de conversión 1.4% (baja) sobre 6,820 clicks → el funnel no convierte bien. CPA $20.66. Recortar y revisar landing/oferta.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1878,13 +1980,13 @@
           <t>Mensajes_WHATSAPP_ARRIENDO_2026</t>
         </is>
       </c>
-      <c r="C5" s="28" t="n">
+      <c r="C5" s="20" t="n">
         <v>650</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>0.70612308</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="19" t="n">
         <v>458.98</v>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -1892,18 +1994,18 @@
           <t>actions:onsite_conversion.messaging_conversation_started_7d</t>
         </is>
       </c>
-      <c r="G5" s="20" t="inlineStr">
+      <c r="G5" s="27" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE</t>
         </is>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="19" t="n">
         <v>670</v>
       </c>
-      <c r="I5" s="21" t="n">
+      <c r="I5" s="23" t="n">
         <v>211.02</v>
       </c>
-      <c r="J5" s="29" t="n">
+      <c r="J5" s="31" t="n">
         <v>0.459758595145758</v>
       </c>
       <c r="K5" s="15" t="inlineStr">
@@ -1911,7 +2013,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L5" s="23" t="inlineStr">
+      <c r="L5" s="25" t="inlineStr">
         <is>
           <t>CPR $0.71 excepcional (650 conversaciones WhatsApp). Es un outlier eficiente del MCC - vale la pena duplicar inversión y dejar que escale.</t>
         </is>
@@ -1928,13 +2030,13 @@
           <t>CONVERSIONES_ARRIENDO_LISTA_RECOMPRA</t>
         </is>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="20" t="n">
         <v>180</v>
       </c>
       <c r="D6" s="16" t="n">
         <v>4.37394444</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="19" t="n">
         <v>787.3099999999999</v>
       </c>
       <c r="F6" s="15" t="inlineStr">
@@ -1942,18 +2044,18 @@
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G6" s="24" t="inlineStr">
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="H6" s="19" t="n">
         <v>830</v>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="I6" s="23" t="n">
         <v>42.69000000000005</v>
       </c>
-      <c r="J6" s="29" t="n">
+      <c r="J6" s="31" t="n">
         <v>0.05422260608908824</v>
       </c>
       <c r="K6" s="15" t="inlineStr">
@@ -1961,7 +2063,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L6" s="23" t="inlineStr">
+      <c r="L6" s="25" t="inlineStr">
         <is>
           <t>CPR $4.37 bueno con 180 conversiones web validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
         </is>
@@ -1978,13 +2080,13 @@
           <t>CONVERSIONES_ARRIENDO_USUARIOS_SIN_INQUILINO_V2</t>
         </is>
       </c>
-      <c r="C7" s="28" t="n">
+      <c r="C7" s="20" t="n">
         <v>124</v>
       </c>
       <c r="D7" s="16" t="n">
         <v>4.71532258</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>584.7</v>
       </c>
       <c r="F7" s="15" t="inlineStr">
@@ -1992,18 +2094,18 @@
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G7" s="24" t="inlineStr">
+      <c r="G7" s="22" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="H7" s="19" t="n">
         <v>616</v>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="23" t="n">
         <v>31.29999999999995</v>
       </c>
-      <c r="J7" s="29" t="n">
+      <c r="J7" s="31" t="n">
         <v>0.05353172567128434</v>
       </c>
       <c r="K7" s="15" t="inlineStr">
@@ -2011,7 +2113,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L7" s="23" t="inlineStr">
+      <c r="L7" s="25" t="inlineStr">
         <is>
           <t>CPR $4.72 bueno con 124 conversiones web validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
         </is>
@@ -2028,13 +2130,13 @@
           <t>CONVERSIONES_ARRIENDO_RMKT_2025</t>
         </is>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="20" t="n">
         <v>522</v>
       </c>
       <c r="D8" s="16" t="n">
         <v>5.0641954</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="19" t="n">
         <v>2643.51</v>
       </c>
       <c r="F8" s="15" t="inlineStr">
@@ -2042,18 +2144,18 @@
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G8" s="30" t="inlineStr">
+      <c r="G8" s="32" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="19" t="n">
         <v>2144</v>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="I8" s="23" t="n">
         <v>-499.5100000000002</v>
       </c>
-      <c r="J8" s="31" t="n">
+      <c r="J8" s="33" t="n">
         <v>-0.188957106271586</v>
       </c>
       <c r="K8" s="15" t="inlineStr">
@@ -2061,7 +2163,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L8" s="23" t="inlineStr">
+      <c r="L8" s="25" t="inlineStr">
         <is>
           <t>CPR $5.06 aceptable. 522 conversiones web. Mantener para no romper aprendizaje del algoritmo.</t>
         </is>
@@ -2078,13 +2180,13 @@
           <t>CONVERSIONES_ARRIENDO_INTERESES_2025</t>
         </is>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="20" t="n">
         <v>741</v>
       </c>
       <c r="D9" s="16" t="n">
         <v>5.45124157</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <v>4039.37</v>
       </c>
       <c r="F9" s="15" t="inlineStr">
@@ -2092,18 +2194,18 @@
           <t xml:space="preserve">conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AD - </t>
         </is>
       </c>
-      <c r="G9" s="30" t="inlineStr">
+      <c r="G9" s="32" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H9" s="19" t="n">
         <v>3275</v>
       </c>
-      <c r="I9" s="21" t="n">
+      <c r="I9" s="23" t="n">
         <v>-764.3699999999999</v>
       </c>
-      <c r="J9" s="31" t="n">
+      <c r="J9" s="33" t="n">
         <v>-0.189230003688694</v>
       </c>
       <c r="K9" s="15" t="inlineStr">
@@ -2111,7 +2213,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L9" s="23" t="inlineStr">
+      <c r="L9" s="25" t="inlineStr">
         <is>
           <t>CPR $5.45 aceptable. 741 conversiones web. Mantener para no romper aprendizaje del algoritmo.</t>
         </is>
@@ -2128,13 +2230,13 @@
           <t>CONVERSIONES_AUTO_PLAN_GLOBAL_INTERESES_2025</t>
         </is>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="20" t="n">
         <v>7</v>
       </c>
       <c r="D10" s="16" t="n">
         <v>1.78857143</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="19" t="n">
         <v>12.52</v>
       </c>
       <c r="F10" s="15" t="inlineStr">
@@ -2142,18 +2244,18 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.Lead_Autos_Di</t>
         </is>
       </c>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="G10" s="27" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE</t>
         </is>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="H10" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="I10" s="21" t="n">
+      <c r="I10" s="23" t="n">
         <v>10.48</v>
       </c>
-      <c r="J10" s="29" t="n">
+      <c r="J10" s="31" t="n">
         <v>0.8370607028753995</v>
       </c>
       <c r="K10" s="15" t="inlineStr">
@@ -2161,7 +2263,7 @@
           <t>inactive</t>
         </is>
       </c>
-      <c r="L10" s="23" t="inlineStr">
+      <c r="L10" s="25" t="inlineStr">
         <is>
           <t>CPR $1.79 excepcional (7 conversiones web). Es un outlier eficiente del MCC - vale la pena duplicar inversión y dejar que escale.</t>
         </is>
@@ -2178,13 +2280,13 @@
           <t>Clientes potenciales - Auto</t>
         </is>
       </c>
-      <c r="C11" s="28" t="n">
+      <c r="C11" s="20" t="n">
         <v>289</v>
       </c>
       <c r="D11" s="16" t="n">
         <v>3.05038062</v>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="19" t="n">
         <v>881.5599999999999</v>
       </c>
       <c r="F11" s="15" t="inlineStr">
@@ -2192,18 +2294,18 @@
           <t>actions:leadgen.other</t>
         </is>
       </c>
-      <c r="G11" s="24" t="inlineStr">
+      <c r="G11" s="22" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H11" s="18" t="n">
+      <c r="H11" s="19" t="n">
         <v>1146</v>
       </c>
-      <c r="I11" s="21" t="n">
+      <c r="I11" s="23" t="n">
         <v>264.4400000000001</v>
       </c>
-      <c r="J11" s="29" t="n">
+      <c r="J11" s="31" t="n">
         <v>0.2999682381233269</v>
       </c>
       <c r="K11" s="15" t="inlineStr">
@@ -2211,7 +2313,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L11" s="23" t="inlineStr">
+      <c r="L11" s="25" t="inlineStr">
         <is>
           <t>CPR $3.05 bueno con 289 leads (form) validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
         </is>
@@ -2228,13 +2330,13 @@
           <t>CONVERSIONES_AUTO_INTERESES_2025</t>
         </is>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="20" t="n">
         <v>907</v>
       </c>
       <c r="D12" s="16" t="n">
         <v>3.96775083</v>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="19" t="n">
         <v>3598.75</v>
       </c>
       <c r="F12" s="15" t="inlineStr">
@@ -2242,18 +2344,18 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G12" s="24" t="inlineStr">
+      <c r="G12" s="22" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H12" s="18" t="n">
+      <c r="H12" s="19" t="n">
         <v>4679</v>
       </c>
-      <c r="I12" s="21" t="n">
+      <c r="I12" s="23" t="n">
         <v>1080.25</v>
       </c>
-      <c r="J12" s="29" t="n">
+      <c r="J12" s="31" t="n">
         <v>0.3001736714136853</v>
       </c>
       <c r="K12" s="15" t="inlineStr">
@@ -2261,7 +2363,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L12" s="23" t="inlineStr">
+      <c r="L12" s="25" t="inlineStr">
         <is>
           <t>CPR $3.97 bueno con 907 conversiones web validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
         </is>
@@ -2278,13 +2380,13 @@
           <t>CONVERSIONES_AUTO_RMKT_2025</t>
         </is>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="20" t="n">
         <v>1083</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>4.11855956</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="19" t="n">
         <v>4460.4</v>
       </c>
       <c r="F13" s="15" t="inlineStr">
@@ -2292,18 +2394,18 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G13" s="24" t="inlineStr">
+      <c r="G13" s="22" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H13" s="18" t="n">
+      <c r="H13" s="19" t="n">
         <v>5799</v>
       </c>
-      <c r="I13" s="21" t="n">
+      <c r="I13" s="23" t="n">
         <v>1338.6</v>
       </c>
-      <c r="J13" s="29" t="n">
+      <c r="J13" s="31" t="n">
         <v>0.3001076136669358</v>
       </c>
       <c r="K13" s="15" t="inlineStr">
@@ -2311,7 +2413,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L13" s="23" t="inlineStr">
+      <c r="L13" s="25" t="inlineStr">
         <is>
           <t>CPR $4.12 bueno con 1,083 conversiones web validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
         </is>
@@ -2328,13 +2430,13 @@
           <t>CONVERSIONES_AUTO_INTERESES_PROMOCIONES</t>
         </is>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="20" t="n">
         <v>176</v>
       </c>
       <c r="D14" s="16" t="n">
         <v>4.51539773</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="19" t="n">
         <v>794.71</v>
       </c>
       <c r="F14" s="15" t="inlineStr">
@@ -2342,18 +2444,18 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G14" s="24" t="inlineStr">
+      <c r="G14" s="22" t="inlineStr">
         <is>
           <t>ESCALAR LEVE</t>
         </is>
       </c>
-      <c r="H14" s="18" t="n">
+      <c r="H14" s="19" t="n">
         <v>1033</v>
       </c>
-      <c r="I14" s="21" t="n">
+      <c r="I14" s="23" t="n">
         <v>238.29</v>
       </c>
-      <c r="J14" s="29" t="n">
+      <c r="J14" s="31" t="n">
         <v>0.2998452265606321</v>
       </c>
       <c r="K14" s="15" t="inlineStr">
@@ -2361,7 +2463,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L14" s="23" t="inlineStr">
+      <c r="L14" s="25" t="inlineStr">
         <is>
           <t>CPR $4.52 bueno con 176 conversiones web validados. Subir budget para ganar volumen sin tocar la eficiencia actual.</t>
         </is>
@@ -2378,13 +2480,13 @@
           <t>CONVERSIONES_AUTO_RMKT_PROMOCIONES</t>
         </is>
       </c>
-      <c r="C15" s="28" t="n">
+      <c r="C15" s="20" t="n">
         <v>157</v>
       </c>
       <c r="D15" s="16" t="n">
         <v>5.58904459</v>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="19" t="n">
         <v>877.48</v>
       </c>
       <c r="F15" s="15" t="inlineStr">
@@ -2392,18 +2494,18 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/AUTOS</t>
         </is>
       </c>
-      <c r="G15" s="30" t="inlineStr">
+      <c r="G15" s="32" t="inlineStr">
         <is>
           <t>MANTENER</t>
         </is>
       </c>
-      <c r="H15" s="18" t="n">
+      <c r="H15" s="19" t="n">
         <v>878</v>
       </c>
-      <c r="I15" s="21" t="n">
+      <c r="I15" s="23" t="n">
         <v>0.5199999999999818</v>
       </c>
-      <c r="J15" s="29" t="n">
+      <c r="J15" s="31" t="n">
         <v>0.0005926060992842934</v>
       </c>
       <c r="K15" s="15" t="inlineStr">
@@ -2411,7 +2513,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L15" s="23" t="inlineStr">
+      <c r="L15" s="25" t="inlineStr">
         <is>
           <t>CPR $5.59 aceptable. 157 conversiones web. Mantener para no romper aprendizaje del algoritmo.</t>
         </is>
@@ -2428,13 +2530,13 @@
           <t>Clientes potenciales - Moto</t>
         </is>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C16" s="20" t="n">
         <v>669</v>
       </c>
       <c r="D16" s="16" t="n">
         <v>1.44726457</v>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E16" s="19" t="n">
         <v>968.22</v>
       </c>
       <c r="F16" s="15" t="inlineStr">
@@ -2442,18 +2544,18 @@
           <t>actions:leadgen.other</t>
         </is>
       </c>
-      <c r="G16" s="20" t="inlineStr">
+      <c r="G16" s="27" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE</t>
         </is>
       </c>
-      <c r="H16" s="18" t="n">
+      <c r="H16" s="19" t="n">
         <v>2596</v>
       </c>
-      <c r="I16" s="21" t="n">
+      <c r="I16" s="23" t="n">
         <v>1627.78</v>
       </c>
-      <c r="J16" s="29" t="n">
+      <c r="J16" s="31" t="n">
         <v>1.681208816178141</v>
       </c>
       <c r="K16" s="15" t="inlineStr">
@@ -2461,7 +2563,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L16" s="23" t="inlineStr">
+      <c r="L16" s="25" t="inlineStr">
         <is>
           <t>CPR $1.45 excepcional (669 leads (form)). Es un outlier eficiente del MCC - vale la pena duplicar inversión y dejar que escale.</t>
         </is>
@@ -2478,13 +2580,13 @@
           <t>CONVERSIONES_MOTO_INTERESES_2025</t>
         </is>
       </c>
-      <c r="C17" s="28" t="n">
+      <c r="C17" s="20" t="n">
         <v>256</v>
       </c>
       <c r="D17" s="16" t="n">
         <v>10.33191406</v>
       </c>
-      <c r="E17" s="18" t="n">
+      <c r="E17" s="19" t="n">
         <v>2644.97</v>
       </c>
       <c r="F17" s="15" t="inlineStr">
@@ -2492,18 +2594,18 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/MOTOS</t>
         </is>
       </c>
-      <c r="G17" s="26" t="inlineStr">
+      <c r="G17" s="29" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="H17" s="18" t="n">
+      <c r="H17" s="19" t="n">
         <v>2561</v>
       </c>
-      <c r="I17" s="21" t="n">
+      <c r="I17" s="23" t="n">
         <v>-83.9699999999998</v>
       </c>
-      <c r="J17" s="31" t="n">
+      <c r="J17" s="33" t="n">
         <v>-0.03174705195143983</v>
       </c>
       <c r="K17" s="15" t="inlineStr">
@@ -2511,7 +2613,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L17" s="23" t="inlineStr">
+      <c r="L17" s="25" t="inlineStr">
         <is>
           <t>CPR $10.33 arriba del rango eficiente del producto. Bajar budget y mover el spend a los ad sets que mejor convierten.</t>
         </is>
@@ -2528,13 +2630,13 @@
           <t>CONVERSIONES_MOTO_RMKT_2025</t>
         </is>
       </c>
-      <c r="C18" s="28" t="n">
+      <c r="C18" s="20" t="n">
         <v>312</v>
       </c>
       <c r="D18" s="16" t="n">
         <v>10.69041667</v>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E18" s="19" t="n">
         <v>3335.41</v>
       </c>
       <c r="F18" s="15" t="inlineStr">
@@ -2542,18 +2644,18 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/MOTOS</t>
         </is>
       </c>
-      <c r="G18" s="26" t="inlineStr">
+      <c r="G18" s="29" t="inlineStr">
         <is>
           <t>RECORTAR</t>
         </is>
       </c>
-      <c r="H18" s="18" t="n">
+      <c r="H18" s="19" t="n">
         <v>3230</v>
       </c>
-      <c r="I18" s="21" t="n">
+      <c r="I18" s="23" t="n">
         <v>-105.4099999999999</v>
       </c>
-      <c r="J18" s="31" t="n">
+      <c r="J18" s="33" t="n">
         <v>-0.03160331113716151</v>
       </c>
       <c r="K18" s="15" t="inlineStr">
@@ -2561,7 +2663,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L18" s="23" t="inlineStr">
+      <c r="L18" s="25" t="inlineStr">
         <is>
           <t>CPR $10.69 arriba del rango eficiente del producto. Bajar budget y mover el spend a los ad sets que mejor convierten.</t>
         </is>
@@ -2578,13 +2680,13 @@
           <t>MENSAJES_VIAJES_WHATSAPP_2025</t>
         </is>
       </c>
-      <c r="C19" s="28" t="n">
+      <c r="C19" s="20" t="n">
         <v>784</v>
       </c>
       <c r="D19" s="16" t="n">
         <v>0.66506378</v>
       </c>
-      <c r="E19" s="18" t="n">
+      <c r="E19" s="19" t="n">
         <v>521.41</v>
       </c>
       <c r="F19" s="15" t="inlineStr">
@@ -2592,18 +2694,18 @@
           <t>actions:onsite_conversion.messaging_conversation_started_7d</t>
         </is>
       </c>
-      <c r="G19" s="20" t="inlineStr">
+      <c r="G19" s="27" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE</t>
         </is>
       </c>
-      <c r="H19" s="18" t="n">
+      <c r="H19" s="19" t="n">
         <v>2068</v>
       </c>
-      <c r="I19" s="21" t="n">
+      <c r="I19" s="23" t="n">
         <v>1546.59</v>
       </c>
-      <c r="J19" s="29" t="n">
+      <c r="J19" s="31" t="n">
         <v>2.966168658061795</v>
       </c>
       <c r="K19" s="15" t="inlineStr">
@@ -2611,7 +2713,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L19" s="23" t="inlineStr">
+      <c r="L19" s="25" t="inlineStr">
         <is>
           <t>CPR $0.67 excepcional (784 conversaciones WhatsApp). Es un outlier eficiente del MCC - vale la pena duplicar inversión y dejar que escale.</t>
         </is>
@@ -2628,13 +2730,13 @@
           <t>CONVERSIONES_VIAJES_INTERESES_2025_V2</t>
         </is>
       </c>
-      <c r="C20" s="28" t="n">
+      <c r="C20" s="20" t="n">
         <v>41</v>
       </c>
       <c r="D20" s="16" t="n">
         <v>28.6402439</v>
       </c>
-      <c r="E20" s="18" t="n">
+      <c r="E20" s="19" t="n">
         <v>1174.25</v>
       </c>
       <c r="F20" s="15" t="inlineStr">
@@ -2642,18 +2744,18 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G20" s="27" t="inlineStr">
+      <c r="G20" s="30" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE</t>
         </is>
       </c>
-      <c r="H20" s="18" t="n">
+      <c r="H20" s="19" t="n">
         <v>1035</v>
       </c>
-      <c r="I20" s="21" t="n">
+      <c r="I20" s="23" t="n">
         <v>-139.25</v>
       </c>
-      <c r="J20" s="31" t="n">
+      <c r="J20" s="33" t="n">
         <v>-0.1185863317010858</v>
       </c>
       <c r="K20" s="15" t="inlineStr">
@@ -2661,7 +2763,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L20" s="23" t="inlineStr">
+      <c r="L20" s="25" t="inlineStr">
         <is>
           <t>CPR $28.64 muy alto. $1,174 generaron solo 41 conversiones web. Pausar/recortar y reformular antes de seguir gastando.</t>
         </is>
@@ -2678,13 +2780,13 @@
           <t>CONVERSIONES_VIAJES_RMKT_2025_V2</t>
         </is>
       </c>
-      <c r="C21" s="28" t="n">
+      <c r="C21" s="20" t="n">
         <v>37</v>
       </c>
       <c r="D21" s="16" t="n">
         <v>31.48378378</v>
       </c>
-      <c r="E21" s="18" t="n">
+      <c r="E21" s="19" t="n">
         <v>1164.9</v>
       </c>
       <c r="F21" s="15" t="inlineStr">
@@ -2692,18 +2794,18 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G21" s="27" t="inlineStr">
+      <c r="G21" s="30" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE</t>
         </is>
       </c>
-      <c r="H21" s="18" t="n">
+      <c r="H21" s="19" t="n">
         <v>1027</v>
       </c>
-      <c r="I21" s="21" t="n">
+      <c r="I21" s="23" t="n">
         <v>-137.9000000000001</v>
       </c>
-      <c r="J21" s="31" t="n">
+      <c r="J21" s="33" t="n">
         <v>-0.1183792600223196</v>
       </c>
       <c r="K21" s="15" t="inlineStr">
@@ -2711,7 +2813,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L21" s="23" t="inlineStr">
+      <c r="L21" s="25" t="inlineStr">
         <is>
           <t>CPR $31.48 muy alto. $1,165 generaron solo 37 conversiones web. Pausar/recortar y reformular antes de seguir gastando.</t>
         </is>
@@ -2728,13 +2830,13 @@
           <t>CONVERSIONES_VIAJES_RMKT_PROMOCIONES</t>
         </is>
       </c>
-      <c r="C22" s="28" t="n">
+      <c r="C22" s="20" t="n">
         <v>7</v>
       </c>
       <c r="D22" s="16" t="n">
         <v>34.17285714</v>
       </c>
-      <c r="E22" s="18" t="n">
+      <c r="E22" s="19" t="n">
         <v>239.21</v>
       </c>
       <c r="F22" s="15" t="inlineStr">
@@ -2742,18 +2844,18 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G22" s="27" t="inlineStr">
+      <c r="G22" s="30" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE</t>
         </is>
       </c>
-      <c r="H22" s="18" t="n">
+      <c r="H22" s="19" t="n">
         <v>211</v>
       </c>
-      <c r="I22" s="21" t="n">
+      <c r="I22" s="23" t="n">
         <v>-28.21000000000001</v>
       </c>
-      <c r="J22" s="31" t="n">
+      <c r="J22" s="33" t="n">
         <v>-0.1179298524309185</v>
       </c>
       <c r="K22" s="15" t="inlineStr">
@@ -2761,7 +2863,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L22" s="23" t="inlineStr">
+      <c r="L22" s="25" t="inlineStr">
         <is>
           <t>CPR $34.17 muy alto. $239 generaron solo 7 conversiones web. Pausar/recortar y reformular antes de seguir gastando.</t>
         </is>
@@ -2778,13 +2880,13 @@
           <t>CONVERSIONES_VIAJES_INTERESES_PROMOCIONES</t>
         </is>
       </c>
-      <c r="C23" s="28" t="n">
+      <c r="C23" s="20" t="n">
         <v>5</v>
       </c>
       <c r="D23" s="16" t="n">
         <v>48.606</v>
       </c>
-      <c r="E23" s="18" t="n">
+      <c r="E23" s="19" t="n">
         <v>243.03</v>
       </c>
       <c r="F23" s="15" t="inlineStr">
@@ -2792,18 +2894,18 @@
           <t>conversions:offsite_conversion.fb_pixel_custom.SURA.CO/VIAJE</t>
         </is>
       </c>
-      <c r="G23" s="27" t="inlineStr">
+      <c r="G23" s="30" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE</t>
         </is>
       </c>
-      <c r="H23" s="18" t="n">
+      <c r="H23" s="19" t="n">
         <v>214</v>
       </c>
-      <c r="I23" s="21" t="n">
+      <c r="I23" s="23" t="n">
         <v>-29.03</v>
       </c>
-      <c r="J23" s="31" t="n">
+      <c r="J23" s="33" t="n">
         <v>-0.1194502736287701</v>
       </c>
       <c r="K23" s="15" t="inlineStr">
@@ -2811,7 +2913,7 @@
           <t>active</t>
         </is>
       </c>
-      <c r="L23" s="23" t="inlineStr">
+      <c r="L23" s="25" t="inlineStr">
         <is>
           <t>CPR $48.61 muy alto. $243 generaron solo 5 conversiones web. Pausar/recortar y reformular antes de seguir gastando.</t>
         </is>
@@ -2867,22 +2969,22 @@
           <t>Auto</t>
         </is>
       </c>
-      <c r="B28" s="32" t="n">
+      <c r="B28" s="34" t="n">
         <v>6</v>
       </c>
       <c r="C28" s="5" t="n">
         <v>10625.42</v>
       </c>
-      <c r="D28" s="33" t="n">
+      <c r="D28" s="35" t="n">
         <v>2619</v>
       </c>
-      <c r="E28" s="34" t="n">
+      <c r="E28" s="36" t="n">
         <v>4.057052310042</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>13558</v>
       </c>
-      <c r="G28" s="35" t="n">
+      <c r="G28" s="37" t="n">
         <v>2932.580000000002</v>
       </c>
     </row>
@@ -2892,22 +2994,22 @@
           <t>Moto</t>
         </is>
       </c>
-      <c r="B29" s="32" t="n">
+      <c r="B29" s="34" t="n">
         <v>3</v>
       </c>
       <c r="C29" s="5" t="n">
         <v>6948.599999999999</v>
       </c>
-      <c r="D29" s="33" t="n">
+      <c r="D29" s="35" t="n">
         <v>1237</v>
       </c>
-      <c r="E29" s="34" t="n">
+      <c r="E29" s="36" t="n">
         <v>5.617299919159255</v>
       </c>
       <c r="F29" s="5" t="n">
         <v>8387</v>
       </c>
-      <c r="G29" s="35" t="n">
+      <c r="G29" s="37" t="n">
         <v>1438.400000000001</v>
       </c>
     </row>
@@ -2917,22 +3019,22 @@
           <t>Arriendo</t>
         </is>
       </c>
-      <c r="B30" s="32" t="n">
+      <c r="B30" s="34" t="n">
         <v>5</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>8513.869999999999</v>
       </c>
-      <c r="D30" s="33" t="n">
+      <c r="D30" s="35" t="n">
         <v>2217</v>
       </c>
-      <c r="E30" s="34" t="n">
+      <c r="E30" s="36" t="n">
         <v>3.840266125394677</v>
       </c>
       <c r="F30" s="5" t="n">
         <v>7535</v>
       </c>
-      <c r="G30" s="35" t="n">
+      <c r="G30" s="37" t="n">
         <v>-978.869999999999</v>
       </c>
     </row>
@@ -2942,22 +3044,22 @@
           <t>Viajes</t>
         </is>
       </c>
-      <c r="B31" s="32" t="n">
+      <c r="B31" s="34" t="n">
         <v>5</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>3342.8</v>
       </c>
-      <c r="D31" s="33" t="n">
+      <c r="D31" s="35" t="n">
         <v>874</v>
       </c>
-      <c r="E31" s="34" t="n">
+      <c r="E31" s="36" t="n">
         <v>3.824713958810069</v>
       </c>
       <c r="F31" s="5" t="n">
         <v>4555</v>
       </c>
-      <c r="G31" s="35" t="n">
+      <c r="G31" s="37" t="n">
         <v>1212.2</v>
       </c>
     </row>
@@ -2976,7 +3078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2991,208 +3093,232 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="36" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>Datos base</t>
         </is>
       </c>
-      <c r="B3" s="37" t="inlineStr">
+      <c r="B3" s="39" t="inlineStr">
         <is>
           <t>Performance real del 1-27 abril 2026 cruzado con Sheet Leads CRM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="36" t="inlineStr">
+      <c r="A4" s="38" t="inlineStr">
         <is>
           <t>Constraint 1</t>
         </is>
       </c>
-      <c r="B4" s="37" t="inlineStr">
+      <c r="B4" s="39" t="inlineStr">
         <is>
           <t>Tope por seguro provisto por el cliente (Auto $52.421, Moto $32.642, Arriendo $31.080, Viajes $16.900)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="inlineStr">
+      <c r="A5" s="38" t="inlineStr">
         <is>
           <t>Constraint 2</t>
         </is>
       </c>
-      <c r="B5" s="37" t="inlineStr">
+      <c r="B5" s="39" t="inlineStr">
         <is>
           <t>70-75% del presupuesto en Google (mejor calidad de leads SF según cliente)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="38" t="inlineStr">
         <is>
           <t>Constraint 3</t>
         </is>
       </c>
-      <c r="B6" s="37" t="inlineStr">
+      <c r="B6" s="39" t="inlineStr">
         <is>
           <t>Bing se mantiene en presupuesto del Flow</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="38" t="inlineStr"/>
-      <c r="B7" s="37" t="inlineStr"/>
+      <c r="A7" s="40" t="inlineStr"/>
+      <c r="B7" s="39" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="41" t="inlineStr">
         <is>
           <t>Reglas de clasificación de campañas Google</t>
         </is>
       </c>
-      <c r="B8" s="37" t="inlineStr"/>
+      <c r="B8" s="39" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="38" t="inlineStr">
+        <is>
+          <t>Variables consideradas</t>
+        </is>
+      </c>
+      <c r="B9" s="39" t="inlineStr">
+        <is>
+          <t>CPA + % Lost Budget + Tasa de conversión (conv/clicks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="38" t="inlineStr">
+        <is>
+          <t>Tasa de conversión</t>
+        </is>
+      </c>
+      <c r="B10" s="39" t="inlineStr">
+        <is>
+          <t>Buckets: alta ≥ 8% · media 4-8% · baja &lt; 4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="38" t="inlineStr">
         <is>
           <t>ESCALAR FUERTE (×1.80)</t>
         </is>
       </c>
-      <c r="B9" s="37" t="inlineStr">
-        <is>
-          <t>CPA ≤ $7 y % Lost Budget ≥ 50% — palanca #1</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="36" t="inlineStr">
+      <c r="B11" s="39" t="inlineStr">
+        <is>
+          <t>CPA ≤ $7 + Lost Budget ≥ 50% + tasa conv alta o media — palanca #1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="38" t="inlineStr">
         <is>
           <t>ESCALAR (×1.40)</t>
         </is>
       </c>
-      <c r="B10" s="37" t="inlineStr">
-        <is>
-          <t>CPA ≤ $10 y % Lost Budget ≥ 30%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="36" t="inlineStr">
+      <c r="B12" s="39" t="inlineStr">
+        <is>
+          <t>CPA ≤ $10 + Lost Budget ≥ 30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="38" t="inlineStr">
         <is>
           <t>ESCALAR LEVE (×1.20)</t>
         </is>
       </c>
-      <c r="B11" s="37" t="inlineStr">
-        <is>
-          <t>CPA ≤ $10 y % Lost Budget ≥ 10%</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="36" t="inlineStr">
-        <is>
-          <t>ESCALAR MODERADO (×1.20)</t>
-        </is>
-      </c>
-      <c r="B12" s="37" t="inlineStr">
-        <is>
-          <t>CPA ≤ $15 y % Lost Budget ≥ 50%</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="36" t="inlineStr">
+      <c r="B13" s="39" t="inlineStr">
+        <is>
+          <t>CPA ≤ $10 + Lost Budget ≥ 10% + tasa conv alta o media</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="38" t="inlineStr">
+        <is>
+          <t>ESCALAR MODERADO (×1.15)</t>
+        </is>
+      </c>
+      <c r="B14" s="39" t="inlineStr">
+        <is>
+          <t>CPA $10-15 + Lost Budget ≥ 50% + tasa conv alta (solo si convierte bien)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="38" t="inlineStr">
         <is>
           <t>RECORTAR (×0.65)</t>
         </is>
       </c>
-      <c r="B13" s="37" t="inlineStr">
-        <is>
-          <t>CPA entre $15 y $25</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="36" t="inlineStr">
+      <c r="B15" s="39" t="inlineStr">
+        <is>
+          <t>CPA $15-25, o tasa conv baja con CPA &gt; $10</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="38" t="inlineStr">
         <is>
           <t>RECORTAR FUERTE (×0.40)</t>
         </is>
       </c>
-      <c r="B14" s="37" t="inlineStr">
+      <c r="B16" s="39" t="inlineStr">
         <is>
           <t>CPA &gt; $25</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="36" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="38" t="inlineStr">
         <is>
           <t>MANTENER (×1.00)</t>
         </is>
       </c>
-      <c r="B15" s="37" t="inlineStr">
-        <is>
-          <t>Resto</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="38" t="inlineStr"/>
-      <c r="B16" s="37" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="36" t="inlineStr">
+      <c r="B17" s="39" t="inlineStr">
+        <is>
+          <t>Resto - se monitorea sin tocar</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="40" t="inlineStr"/>
+      <c r="B18" s="39" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="38" t="inlineStr">
         <is>
           <t>Ajuste fino</t>
         </is>
       </c>
-      <c r="B17" s="37" t="inlineStr">
+      <c r="B19" s="39" t="inlineStr">
         <is>
           <t>Después del factor inicial, los presupuestos de Google se reescalan proporcionalmente para alcanzar exactamente el 72% del total por seguro.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="38" t="inlineStr"/>
-      <c r="B18" s="37" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="39" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="40" t="inlineStr"/>
+      <c r="B20" s="39" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="41" t="inlineStr">
         <is>
           <t>Limitaciones honestas</t>
         </is>
       </c>
-      <c r="B19" s="37" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="36" t="inlineStr">
+      <c r="B21" s="39" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="38" t="inlineStr">
         <is>
           <t>Meta</t>
         </is>
       </c>
-      <c r="B20" s="37" t="inlineStr">
+      <c r="B22" s="39" t="inlineStr">
         <is>
           <t>Detalle por ad set requiere CSV exportado del Ads Manager (Reports → Export Reports). Esta propuesta optimiza Meta a nivel seguro.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="36" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="38" t="inlineStr">
         <is>
           <t>Bing</t>
         </is>
       </c>
-      <c r="B21" s="37" t="inlineStr">
+      <c r="B23" s="39" t="inlineStr">
         <is>
           <t>No se modificó (sin acceso desde el extractor).</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="36" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="38" t="inlineStr">
         <is>
           <t>Estacionalidad</t>
         </is>
       </c>
-      <c r="B22" s="37" t="inlineStr">
+      <c r="B24" s="39" t="inlineStr">
         <is>
           <t>Asume ritmo similar a abril. Si hay cambios estacionales, ajustar.</t>
         </is>

</xml_diff>